<commit_message>
📊 Horarios actualizados Línea 141 - 1569
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:42:21</t>
+          <t>Última actualización: 02:03:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>00:42:21</t>
+          <t>02:03:25</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:13</t>
+          <t>02:56</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>31</v>
+        <v>53</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,12 +498,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>00:42:21</t>
+          <t>02:03:25</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>01:59</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -512,9 +512,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>77</v>
+        <v>105</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>02:03:25</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>03:51</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>83_ESC 6_ALUAR</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>108</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -544,7 +569,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:42:21</t>
+          <t>Última actualización: 02:03:25</t>
         </is>
       </c>
     </row>
@@ -585,12 +610,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>00:42:21</t>
+          <t>02:03:25</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:13</t>
+          <t>02:56</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -599,7 +624,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>31</v>
+        <v>53</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -631,7 +656,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:42:21</t>
+          <t>Última actualización: 02:03:25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1570
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:03:25</t>
+          <t>Última actualización: 02:55:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -473,7 +473,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:03:25</t>
+          <t>02:55:59</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,12 +498,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:03:25</t>
+          <t>02:55:59</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>03:47</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>105</v>
+        <v>52</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,12 +523,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:03:25</t>
+          <t>02:55:59</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>03:51</t>
+          <t>03:50</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -537,9 +537,84 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>108</v>
+        <v>55</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>02:55:59</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>04:31</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>96</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>02:55:59</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>04:47</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>112</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>02:55:59</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>113</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -556,7 +631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -569,14 +644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:03:25</t>
+          <t>Última actualización: 02:55:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 2</t>
         </is>
       </c>
     </row>
@@ -610,7 +685,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:03:25</t>
+          <t>02:55:59</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -624,9 +699,34 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>53</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>02:55:59</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>113</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -656,7 +756,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:03:25</t>
+          <t>Última actualización: 02:55:59</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1571
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:55:59</t>
+          <t>Última actualización: 03:34:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:55:59</t>
+          <t>03:34:49</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:56</t>
+          <t>03:48</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:55:59</t>
+          <t>03:34:49</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03:47</t>
+          <t>04:01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>02:55:59</t>
+          <t>03:34:49</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>03:50</t>
+          <t>04:46</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>83_ESC 6_ALUAR</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>02:55:59</t>
+          <t>03:34:49</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:31</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>02:55:59</t>
+          <t>03:34:49</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>05:11</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>112</v>
+        <v>97</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,23 +598,48 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>02:55:59</t>
+          <t>03:34:49</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>03:34:49</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>05:31</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>117</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -631,7 +656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -644,14 +669,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:55:59</t>
+          <t>Última actualización: 03:34:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 1</t>
         </is>
       </c>
     </row>
@@ -685,48 +710,23 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:55:59</t>
+          <t>03:34:49</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>02:56</t>
+          <t>04:46</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>72</v>
       </c>
       <c r="E6" t="inlineStr">
-        <is>
-          <t>LP1912</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>02:55:59</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>04:48</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>215A_EL PATO</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>113</v>
-      </c>
-      <c r="E7" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -756,7 +756,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:55:59</t>
+          <t>Última actualización: 03:34:49</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1572
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:34:49</t>
+          <t>Última actualización: 04:23:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:34:49</t>
+          <t>04:23:04</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03:48</t>
+          <t>04:47</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>03:34:49</t>
+          <t>04:23:04</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:01</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03:34:49</t>
+          <t>04:23:04</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04:46</t>
+          <t>05:12</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:34:49</t>
+          <t>04:23:04</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>79</v>
+        <v>59</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>03:34:49</t>
+          <t>04:23:04</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:11</t>
+          <t>05:32</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>97</v>
+        <v>69</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>03:34:49</t>
+          <t>04:23:04</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:51</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>108</v>
+        <v>88</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,23 +623,98 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>03:34:49</t>
+          <t>04:23:04</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>05:31</t>
+          <t>05:52</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>117</v>
+        <v>89</v>
       </c>
       <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04:23:04</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>98</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>04:23:04</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:04</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>101</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>04:23:04</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>108</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -656,7 +731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -669,14 +744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:34:49</t>
+          <t>Última actualización: 04:23:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 2</t>
         </is>
       </c>
     </row>
@@ -710,12 +785,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03:34:49</t>
+          <t>04:23:04</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:46</t>
+          <t>04:47</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -724,9 +799,34 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>72</v>
+        <v>24</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>04:23:04</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>06:11</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>108</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -756,7 +856,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:34:49</t>
+          <t>Última actualización: 04:23:04</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1573
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:23:04</t>
+          <t>Última actualización: 04:52:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:23:04</t>
+          <t>04:52:39</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:23:04</t>
+          <t>04:52:39</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:11</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:23:04</t>
+          <t>04:52:39</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:12</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:23:04</t>
+          <t>04:52:39</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:31</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:23:04</t>
+          <t>04:52:39</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:32</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>52</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:23:04</t>
+          <t>04:52:39</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:51</t>
+          <t>05:52</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>88</v>
+        <v>60</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:23:04</t>
+          <t>04:52:39</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>05:52</t>
+          <t>06:00</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:23:04</t>
+          <t>04:52:39</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:03</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>98</v>
+        <v>71</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:23:04</t>
+          <t>04:52:39</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:04</t>
+          <t>06:10</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>101</v>
+        <v>78</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,23 +698,148 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:23:04</t>
+          <t>04:52:39</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:11</t>
+          <t>06:24</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>92</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>04:52:39</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>06:27</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>95</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>04:52:39</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>98</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>04:52:39</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>06:31</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>99</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>04:52:39</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>107</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>04:52:39</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>06:50</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>108</v>
-      </c>
-      <c r="E15" t="inlineStr">
+      <c r="D20" t="n">
+        <v>118</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -744,7 +869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:23:04</t>
+          <t>Última actualización: 04:52:39</t>
         </is>
       </c>
     </row>
@@ -785,21 +910,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:23:04</t>
+          <t>04:52:39</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:47</t>
+          <t>06:10</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>24</v>
+        <v>78</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -810,12 +935,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:23:04</t>
+          <t>04:52:39</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06:11</t>
+          <t>06:50</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -824,7 +949,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -856,7 +981,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:23:04</t>
+          <t>Última actualización: 04:52:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1574
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:52:39</t>
+          <t>Última actualización: 05:21:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>05:32</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:11</t>
+          <t>05:42</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:44</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:31</t>
+          <t>05:52</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:04</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05:52</t>
+          <t>06:11</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:00</t>
+          <t>06:24</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:03</t>
+          <t>06:27</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:10</t>
+          <t>06:31</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:24</t>
+          <t>06:31</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>92</v>
+        <v>70</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:27</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>95</v>
+        <v>78</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:51</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>98</v>
+        <v>90</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:31</t>
+          <t>07:01</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>07:01</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,23 +823,73 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>06:50</t>
+          <t>07:04</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>05:21:26</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>07:06</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>105</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>05:21:26</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>07:13</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>112</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -856,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -869,14 +919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:52:39</t>
+          <t>Última actualización: 05:21:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -910,12 +960,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>06:10</t>
+          <t>06:11</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -924,7 +974,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>78</v>
+        <v>50</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -935,12 +985,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04:52:39</t>
+          <t>05:21:26</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>06:50</t>
+          <t>06:51</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -949,9 +999,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>118</v>
+        <v>90</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>05:21:26</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:06</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>105</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -981,7 +1056,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:52:39</t>
+          <t>Última actualización: 05:21:26</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1575
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:21:26</t>
+          <t>Última actualización: 05:56:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -473,21 +473,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>05:32</t>
+          <t>06:03</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -498,21 +498,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>05:42</t>
+          <t>06:11</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -523,21 +523,21 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>06:18</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -548,21 +548,21 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>05:52</t>
+          <t>06:24</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:04</t>
+          <t>06:27</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -598,21 +598,21 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:11</t>
+          <t>06:31</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,21 +623,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06:24</t>
+          <t>06:31</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:27</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>66</v>
+        <v>43</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:31</t>
+          <t>06:51</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>70</v>
+        <v>55</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:31</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>07:01</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>06:51</t>
+          <t>07:04</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:01</t>
+          <t>07:06</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,21 +798,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:01</t>
+          <t>07:13</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>100</v>
+        <v>77</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:04</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07:06</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,23 +873,73 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>07:13</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>112</v>
+        <v>100</v>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>05:56:34</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>07:43</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>107</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>05:56:34</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>113</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -919,7 +969,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:21:26</t>
+          <t>Última actualización: 05:56:34</t>
         </is>
       </c>
     </row>
@@ -960,7 +1010,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -974,7 +1024,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -985,7 +1035,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -999,7 +1049,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>90</v>
+        <v>55</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1010,7 +1060,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:21:26</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1024,7 +1074,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>105</v>
+        <v>70</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1043,7 +1093,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1056,14 +1106,66 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:21:26</t>
+          <t>Última actualización: 05:56:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 0</t>
+          <t>Total filas: 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Hora_Scrap</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hora_Llegada</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Linea</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Minutos</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Parada</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>05:56:34</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>07:27</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>91</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1576
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:56:34</t>
+          <t>Última actualización: 06:25:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -573,21 +573,21 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:25:24</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>06:27</t>
+          <t>06:25</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -603,16 +603,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>06:31</t>
+          <t>06:27</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -623,7 +623,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:25:24</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -633,11 +633,11 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -648,21 +648,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:25:24</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>06:31</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>43</v>
+        <v>6</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,21 +673,21 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:25:24</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>06:51</t>
+          <t>06:31</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>55</v>
+        <v>6</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:25:24</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>63</v>
+        <v>14</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -723,21 +723,21 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:25:24</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>07:01</t>
+          <t>06:46</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -748,21 +748,21 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:25:24</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:04</t>
+          <t>06:51</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>68</v>
+        <v>26</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -773,21 +773,21 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:25:24</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>07:06</t>
+          <t>06:56</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -803,16 +803,16 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>07:13</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:25:24</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>93</v>
+        <v>36</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:25:24</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:04</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>100</v>
+        <v>39</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -878,16 +878,16 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:06</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,21 +898,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:25:24</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>07:43</t>
+          <t>07:07</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>107</v>
+        <v>42</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -928,18 +928,318 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>07:13</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>77</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>06:25:24</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>07:14</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>49</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>06:25:24</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>56</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>06:25:24</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>07:29</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>64</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>06:25:24</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>71</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>05:56:34</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>100</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>06:25:24</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>72</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>05:56:34</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>07:43</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>107</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>06:25:24</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>79</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>06:25:24</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t>07:49</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>113</v>
-      </c>
-      <c r="E24" t="inlineStr">
+      <c r="D33" t="n">
+        <v>84</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>06:25:24</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>07:59</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>94</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>06:25:24</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>08:14</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>109</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>06:25:24</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>114</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -956,7 +1256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -969,14 +1269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:56:34</t>
+          <t>Última actualización: 06:25:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1335,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:25:24</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1049,7 +1349,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>55</v>
+        <v>26</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -1077,6 +1377,56 @@
         <v>70</v>
       </c>
       <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06:25:24</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>07:07</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>42</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>06:25:24</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>07:21</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>56</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1093,7 +1443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1106,14 +1456,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:56:34</t>
+          <t>Última actualización: 06:25:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -1166,6 +1516,81 @@
       <c r="E6" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>06:25:24</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:28</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>63</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:25:24</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>08:10</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>105</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06:25:24</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:23</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>118</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1577
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:25:25</t>
+          <t>Última actualización: 06:53:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -773,12 +773,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>06:25:24</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>06:56</t>
+          <t>06:53</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>31</v>
+        <v>0</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,12 +798,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:25:24</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>06:56</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -812,7 +812,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:25:24</t>
+          <t>05:56:34</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>07:01</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>36</v>
+        <v>63</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:25:24</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>07:04</t>
+          <t>07:01</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>39</v>
+        <v>8</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,21 +873,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>07:06</t>
+          <t>07:04</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>70</v>
+        <v>11</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,12 +898,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>06:25:24</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>07:07</t>
+          <t>07:06</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>42</v>
+        <v>13</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,21 +923,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:25:24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>07:13</t>
+          <t>07:07</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>77</v>
+        <v>42</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -948,12 +948,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>06:25:24</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>07:14</t>
+          <t>07:13</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -978,16 +978,16 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:14</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,21 +998,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>06:25:24</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>64</v>
+        <v>28</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,21 +1023,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06:25:24</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:24</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>71</v>
+        <v>31</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,21 +1048,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>100</v>
+        <v>36</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>06:25:24</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:33</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>07:43</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>107</v>
+        <v>43</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:25:24</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>79</v>
+        <v>43</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1153,16 +1153,16 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>07:49</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:25:24</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:43</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>94</v>
+        <v>50</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>08:14</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>109</v>
+        <v>79</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,23 +1223,223 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>06:25:24</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>07:49</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>56</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>06:53:33</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>07:59</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>66</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>06:53:33</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>08:03</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>70</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>06:53:33</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>08:08</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>75</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>06:53:33</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>08:14</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>81</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>06:53:33</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
           <t>08:19</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>114</v>
-      </c>
-      <c r="E36" t="inlineStr">
+      <c r="D41" t="n">
+        <v>86</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>06:53:33</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>08:34</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>101</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>06:53:33</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>115</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>06:53:33</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>08:51</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>118</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1256,7 +1456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1269,14 +1469,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:25:25</t>
+          <t>Última actualización: 06:53:33</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1360,7 +1560,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1374,7 +1574,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>70</v>
+        <v>13</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1410,7 +1610,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>06:25:24</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1424,9 +1624,59 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>56</v>
+        <v>28</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06:53:33</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:34</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>101</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>06:53:33</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>115</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1456,7 +1706,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:25:25</t>
+          <t>Última actualización: 06:53:33</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1747,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>05:56:34</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1511,7 +1761,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>91</v>
+        <v>34</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1547,7 +1797,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>06:25:24</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1561,7 +1811,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>105</v>
+        <v>77</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1572,7 +1822,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>06:25:24</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1586,7 +1836,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>118</v>
+        <v>90</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1578
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:53:33</t>
+          <t>Última actualización: 07:16:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 48</t>
         </is>
       </c>
     </row>
@@ -1023,12 +1023,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>07:24</t>
+          <t>07:23</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1053,16 +1053,16 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>07:29</t>
+          <t>07:24</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>07:33</t>
+          <t>07:29</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1103,16 +1103,16 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:33</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,21 +1148,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>06:25:24</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>72</v>
+        <v>20</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>07:43</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1203,16 +1203,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>07:44</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,21 +1223,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>07:49</t>
+          <t>07:41</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:43</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>66</v>
+        <v>27</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>06:25:24</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>08:03</t>
+          <t>07:44</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>08:08</t>
+          <t>07:49</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>75</v>
+        <v>33</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>08:14</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>81</v>
+        <v>43</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>86</v>
+        <v>47</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>08:34</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>101</v>
+        <v>50</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1403,16 +1403,16 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>08:48</t>
+          <t>08:08</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>115</v>
+        <v>75</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,23 +1423,248 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>07:16:54</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>08:14</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>58</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>07:16:54</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>08:19</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>63</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>07:16:54</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>08:29</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>73</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>07:16:54</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>77</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
           <t>06:53:33</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>08:34</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>101</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>07:16:54</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>08:47</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>91</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>06:53:33</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>115</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>07:16:54</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
         <is>
           <t>08:51</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D44" t="n">
+      <c r="D51" t="n">
+        <v>95</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>07:16:54</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>08:59</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>103</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>07:16:54</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
         <v>118</v>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1456,7 +1681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1469,14 +1694,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:53:33</t>
+          <t>Última actualización: 07:16:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -1635,12 +1860,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>08:34</t>
+          <t>08:33</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1649,7 +1874,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1665,18 +1890,93 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
+          <t>08:34</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>101</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07:16:54</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>08:47</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>91</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>06:53:33</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>08:48</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D14" t="n">
         <v>115</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>07:16:54</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>08:59</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>103</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1693,7 +1993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1706,14 +2006,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:53:33</t>
+          <t>Última actualización: 07:16:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -1747,7 +2047,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1761,7 +2061,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -1822,23 +2122,73 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>07:16:54</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:11</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>55</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>06:53:33</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>08:23</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D10" t="n">
         <v>90</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>07:16:54</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:27</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>71</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1579
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:16:54</t>
+          <t>Última actualización: 07:48:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 48</t>
+          <t>Total filas: 63</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>07:49</t>
+          <t>07:48</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1328,16 +1328,16 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:49</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>08:03</t>
+          <t>07:50</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>47</v>
+        <v>2</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1378,16 +1378,16 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>08:06</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,12 +1398,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>08:08</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1412,7 +1412,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>75</v>
+        <v>11</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>08:14</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>08:01</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>63</v>
+        <v>13</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>08:29</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>73</v>
+        <v>15</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1503,16 +1503,16 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>08:33</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1528,16 +1528,16 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>08:34</t>
+          <t>08:08</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>101</v>
+        <v>75</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>08:47</t>
+          <t>08:14</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>91</v>
+        <v>26</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>08:48</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>115</v>
+        <v>31</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>08:51</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>95</v>
+        <v>33</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1628,16 +1628,16 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>08:59</t>
+          <t>08:29</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>103</v>
+        <v>73</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,23 +1648,398 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>42</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
           <t>07:16:54</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>77</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>08:34</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>46</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>07:16:54</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>08:47</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>91</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>60</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>08:51</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>63</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>07:16:54</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>08:59</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>103</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>72</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>75</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>09:05</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>77</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>07:16:54</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
         <is>
           <t>09:14</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C63" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D53" t="n">
+      <c r="D63" t="n">
         <v>118</v>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>87</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>90</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>91</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>106</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>117</v>
+      </c>
+      <c r="E68" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1681,7 +2056,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1694,14 +2069,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:16:54</t>
+          <t>Última actualización: 07:48:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -1885,7 +2260,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1899,7 +2274,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>101</v>
+        <v>46</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1935,7 +2310,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1949,7 +2324,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>115</v>
+        <v>60</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1977,6 +2352,56 @@
         <v>103</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>72</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>91</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1993,7 +2418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2006,14 +2431,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:16:54</t>
+          <t>Última actualización: 07:48:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -2147,50 +2572,125 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>08:23</t>
+          <t>08:15</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>90</v>
+        <v>27</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>06:53:33</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:23</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>90</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08:24</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>36</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>07:16:54</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>08:27</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D13" t="n">
         <v>71</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>08:52</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>64</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1580
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E68"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:48:06</t>
+          <t>Última actualización: 08:02:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 63</t>
+          <t>Total filas: 72</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>08:03</t>
+          <t>08:02</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>08:06</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,12 +1523,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>06:53:33</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>08:08</t>
+          <t>08:06</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>06:53:33</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>08:14</t>
+          <t>08:08</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>26</v>
+        <v>75</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>08:19</t>
+          <t>08:14</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>31</v>
+        <v>12</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:19</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1623,21 +1623,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>08:29</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>73</v>
+        <v>19</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,12 +1648,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>08:29</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1662,7 +1662,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>42</v>
+        <v>27</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,21 +1673,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>08:33</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>77</v>
+        <v>42</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,12 +1698,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>08:34</t>
+          <t>08:33</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -1712,7 +1712,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>46</v>
+        <v>77</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>08:47</t>
+          <t>08:34</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>91</v>
+        <v>32</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>08:48</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>08:51</t>
+          <t>08:47</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>63</v>
+        <v>91</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>08:59</t>
+          <t>08:48</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>103</v>
+        <v>46</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:51</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>09:03</t>
+          <t>08:59</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>75</v>
+        <v>57</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1878,16 +1878,16 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>09:05</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>118</v>
+        <v>58</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1928,16 +1928,16 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>87</v>
+        <v>75</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1953,16 +1953,16 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>09:05</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,21 +1973,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:13</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>106</v>
+        <v>71</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,23 +2023,248 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t>08:02:29</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>09:14</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>72</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
           <t>07:48:06</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>87</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>90</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>08:02:29</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>09:19</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>77</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>08:02:29</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>09:33</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>91</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>08:02:29</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>92</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>08:02:29</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>102</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
         <is>
           <t>09:45</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D68" t="n">
+      <c r="D75" t="n">
         <v>117</v>
       </c>
-      <c r="E68" t="inlineStr">
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>08:02:29</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>109</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>08:02:29</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>114</v>
+      </c>
+      <c r="E77" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2069,7 +2294,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:48:06</t>
+          <t>Última actualización: 08:02:29</t>
         </is>
       </c>
     </row>
@@ -2260,7 +2485,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -2274,7 +2499,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -2310,7 +2535,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -2324,7 +2549,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -2335,7 +2560,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2349,7 +2574,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>103</v>
+        <v>57</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2385,7 +2610,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2399,7 +2624,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2418,7 +2643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2431,14 +2656,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:48:06</t>
+          <t>Última actualización: 08:02:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 11</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2797,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2586,7 +2811,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>27</v>
+        <v>13</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2647,12 +2872,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>08:27</t>
+          <t>08:25</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2661,7 +2886,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2672,25 +2897,75 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
+          <t>08:27</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>71</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:02:29</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>08:52</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>64</v>
-      </c>
-      <c r="E14" t="inlineStr">
+      <c r="D15" t="n">
+        <v>50</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08:02:29</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>114</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1581
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E77"/>
+  <dimension ref="A1:E89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:02:29</t>
+          <t>Última actualización: 08:33:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 72</t>
+          <t>Total filas: 84</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1698,7 +1698,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1712,7 +1712,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>08:34</t>
+          <t>08:33</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1753,16 +1753,16 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:34</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>08:47</t>
+          <t>08:44</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>91</v>
+        <v>11</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,12 +1798,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>08:48</t>
+          <t>08:47</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1812,7 +1812,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1828,16 +1828,16 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>08:51</t>
+          <t>08:48</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>08:59</t>
+          <t>08:51</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>57</v>
+        <v>18</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,12 +1873,12 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:59</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -1887,7 +1887,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1908,11 +1908,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,12 +1923,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>09:03</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>09:05</t>
+          <t>09:01</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>77</v>
+        <v>28</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,21 +1973,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>09:07</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>09:13</t>
+          <t>09:05</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2028,16 +2028,16 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>09:13</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>09:14</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>90</v>
+        <v>41</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>09:33</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>91</v>
+        <v>43</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>102</v>
+        <v>45</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>09:19</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>117</v>
+        <v>77</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>09:51</t>
+          <t>09:29</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>109</v>
+        <v>56</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2253,18 +2253,318 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
+          <t>09:33</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>91</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>09:34</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>61</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>09:36</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>63</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>09:44</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>71</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>07:48:06</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>117</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>09:49</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>76</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>09:51</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>78</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>09:52</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>79</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
           <t>09:56</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D77" t="n">
-        <v>114</v>
-      </c>
-      <c r="E77" t="inlineStr">
+      <c r="D85" t="n">
+        <v>83</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>10:03</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>90</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>10:08</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>95</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>105</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>119</v>
+      </c>
+      <c r="E89" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2281,7 +2581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2294,14 +2594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:02:29</t>
+          <t>Última actualización: 08:33:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 14</t>
         </is>
       </c>
     </row>
@@ -2460,7 +2760,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2474,7 +2774,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>77</v>
+        <v>0</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -2510,7 +2810,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -2524,7 +2824,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -2560,7 +2860,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2574,7 +2874,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2610,23 +2910,73 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>09:18</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>45</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>08:02:29</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>09:19</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D18" t="n">
         <v>77</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10:03</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>90</v>
+      </c>
+      <c r="E19" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2643,7 +2993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2656,14 +3006,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:02:29</t>
+          <t>Última actualización: 08:33:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 11</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2922,12 +3272,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>08:52</t>
+          <t>08:51</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2936,7 +3286,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2952,20 +3302,120 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
+          <t>08:52</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>50</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>09:55</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>82</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:02:29</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>09:56</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D16" t="n">
+      <c r="D18" t="n">
         <v>114</v>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>97</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>108</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1582
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E89"/>
+  <dimension ref="A1:E99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:33:50</t>
+          <t>Última actualización: 08:51:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 84</t>
+          <t>Total filas: 94</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1858,11 +1858,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>08:59</t>
+          <t>08:51</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,12 +1898,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>08:59</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1912,7 +1912,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>09:01</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>28</v>
+        <v>58</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1973,21 +1973,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>09:03</t>
+          <t>09:01</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>09:05</t>
+          <t>09:03</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>77</v>
+        <v>30</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>09:07</t>
+          <t>09:04</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>65</v>
+        <v>13</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,21 +2048,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>09:13</t>
+          <t>09:05</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>09:14</t>
+          <t>09:07</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>09:13</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2128,16 +2128,16 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:14</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>90</v>
+        <v>24</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2178,16 +2178,16 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>09:19</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>77</v>
+        <v>26</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2228,16 +2228,16 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>09:29</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>09:33</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,21 +2273,21 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:19</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>61</v>
+        <v>28</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>09:36</t>
+          <t>09:29</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>63</v>
+        <v>38</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:33</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>71</v>
+        <v>91</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>117</v>
+        <v>43</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,21 +2373,21 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>09:49</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>76</v>
+        <v>43</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2403,16 +2403,16 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>09:51</t>
+          <t>09:36</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>09:52</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>79</v>
+        <v>50</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2453,16 +2453,16 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>10:03</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>90</v>
+        <v>54</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2503,16 +2503,16 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>10:08</t>
+          <t>09:49</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>10:18</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>105</v>
+        <v>60</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2553,18 +2553,268 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
+          <t>09:52</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>79</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>08:51:02</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>65</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>10:03</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>90</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>08:51:02</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>73</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>10:08</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>95</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>08:51:02</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>80</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>105</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>08:51:02</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>10:19</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>88</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
           <t>10:32</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C97" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D89" t="n">
+      <c r="D97" t="n">
         <v>119</v>
       </c>
-      <c r="E89" t="inlineStr">
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>08:51:02</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>10:33</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>102</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>08:51:02</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>113</v>
+      </c>
+      <c r="E99" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2581,7 +2831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2594,14 +2844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:33:50</t>
+          <t>Última actualización: 08:51:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 14</t>
+          <t>Total filas: 15</t>
         </is>
       </c>
     </row>
@@ -2885,7 +3135,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2899,7 +3149,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>72</v>
+        <v>9</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -2935,7 +3185,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -2949,7 +3199,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>77</v>
+        <v>28</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -2977,6 +3227,31 @@
         <v>90</v>
       </c>
       <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>08:51:02</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>73</v>
+      </c>
+      <c r="E20" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2993,7 +3268,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3006,14 +3281,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:33:50</t>
+          <t>Última actualización: 08:51:02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3572,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3311,7 +3586,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -3347,7 +3622,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3361,7 +3636,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>114</v>
+        <v>65</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -3397,23 +3672,73 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>08:51:02</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>80</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>08:33:50</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>10:21</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D20" t="n">
+      <c r="D21" t="n">
         <v>108</v>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>08:51:02</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>10:22</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>91</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1583
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E99"/>
+  <dimension ref="A1:E110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:51:02</t>
+          <t>Última actualización: 09:25:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 94</t>
+          <t>Total filas: 105</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>09:29</t>
+          <t>09:25</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>09:33</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>91</v>
+        <v>1</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2353,16 +2353,16 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:29</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,12 +2373,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>09:34</t>
+          <t>09:33</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>43</v>
+        <v>8</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>09:36</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>63</v>
+        <v>9</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2428,16 +2428,16 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:34</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2453,16 +2453,16 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>09:44</t>
+          <t>09:36</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2478,16 +2478,16 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>09:49</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>09:51</t>
+          <t>09:44</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>09:52</t>
+          <t>09:45</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>79</v>
+        <v>20</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,21 +2573,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:48</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2603,16 +2603,16 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>10:03</t>
+          <t>09:49</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>90</v>
+        <v>76</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>10:04</t>
+          <t>09:51</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>73</v>
+        <v>26</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2653,16 +2653,16 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>10:08</t>
+          <t>09:52</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>80</v>
+        <v>31</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>10:18</t>
+          <t>10:03</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>105</v>
+        <v>38</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>10:19</t>
+          <t>10:03</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,21 +2748,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>10:32</t>
+          <t>10:04</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>119</v>
+        <v>39</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>10:33</t>
+          <t>10:08</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2803,18 +2803,293 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>80</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>105</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>09:25:12</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>10:19</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>54</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>08:33:50</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>10:32</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>119</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>09:25:12</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>10:33</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>68</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>09:25:12</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
           <t>10:44</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C104" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D99" t="n">
-        <v>113</v>
-      </c>
-      <c r="E99" t="inlineStr">
+      <c r="D104" t="n">
+        <v>79</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>09:25:12</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>92</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>09:25:12</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>97</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>09:25:12</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>103</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>09:25:12</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>114</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>09:25:12</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>11:21</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>116</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>09:25:12</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>11:22</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>117</v>
+      </c>
+      <c r="E110" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2831,7 +3106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2844,14 +3119,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:51:02</t>
+          <t>Última actualización: 09:25:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 15</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3235,7 +3510,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3249,9 +3524,34 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>73</v>
+        <v>39</v>
       </c>
       <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>09:25:12</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>114</v>
+      </c>
+      <c r="E21" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3268,7 +3568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3281,14 +3581,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:51:02</t>
+          <t>Última actualización: 09:25:12</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -3647,37 +3947,37 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>10:10</t>
+          <t>10:02</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>10:10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3686,7 +3986,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>80</v>
+        <v>97</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -3697,21 +3997,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>10:21</t>
+          <t>10:11</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>108</v>
+        <v>46</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3722,23 +4022,48 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>10:21</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>108</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>09:25:12</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>10:22</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>91</v>
-      </c>
-      <c r="E22" t="inlineStr">
+      <c r="D23" t="n">
+        <v>57</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1584
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E110"/>
+  <dimension ref="A1:E131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:25:12</t>
+          <t>Última actualización: 10:25:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 105</t>
+          <t>Total filas: 126</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>10:32</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>119</v>
+        <v>0</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,21 +2898,21 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>10:33</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>68</v>
+        <v>0</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:32</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>79</v>
+        <v>7</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2948,21 +2948,21 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>10:57</t>
+          <t>10:33</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>92</v>
+        <v>8</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>11:02</t>
+          <t>10:33</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>97</v>
+        <v>8</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3003,16 +3003,16 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>10:33</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>103</v>
+        <v>68</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,21 +3023,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>11:19</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>114</v>
+        <v>18</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3053,16 +3053,16 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>11:21</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>116</v>
+        <v>79</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,23 +3073,548 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>10:48</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>23</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>25</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>31</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>31</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
           <t>09:25:12</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr">
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>92</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>09:25:12</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>97</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>11:03</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>38</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>11:05</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>40</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>11:07</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>42</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>09:25:12</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>11:08</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D119" t="n">
+        <v>103</v>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>11:18</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>53</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>09:25:12</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>114</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>55</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>09:25:12</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>11:21</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>116</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>09:25:12</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
         <is>
           <t>11:22</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
+      <c r="C124" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D110" t="n">
+      <c r="D124" t="n">
         <v>117</v>
       </c>
-      <c r="E110" t="inlineStr">
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>11:32</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>67</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>79</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>85</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>90</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>12:03</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>98</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>12:19</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>114</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>12:21</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>116</v>
+      </c>
+      <c r="E131" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3106,7 +3631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3119,14 +3644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:25:12</t>
+          <t>Última actualización: 10:25:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -3535,23 +4060,98 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11:18</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>53</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>09:25:12</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>11:19</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D21" t="n">
+      <c r="D22" t="n">
         <v>114</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>11:32</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>67</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>79</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3568,7 +4168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3581,14 +4181,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:25:12</t>
+          <t>Última actualización: 10:25:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -4066,6 +4666,56 @@
       <c r="E23" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>73</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>90</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1585
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E131"/>
+  <dimension ref="A1:E151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:25:57</t>
+          <t>Última actualización: 10:59:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 126</t>
+          <t>Total filas: 146</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2233,11 +2233,11 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3198,21 +3198,21 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>11:02</t>
+          <t>10:59</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>11:03</t>
+          <t>11:01</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>11:05</t>
+          <t>11:02</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>11:07</t>
+          <t>11:02</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>42</v>
+        <v>97</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>11:08</t>
+          <t>11:03</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>103</v>
+        <v>4</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3328,16 +3328,16 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>11:18</t>
+          <t>11:05</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>11:19</t>
+          <t>11:07</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>114</v>
+        <v>42</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>11:20</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>11:21</t>
+          <t>11:18</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>116</v>
+        <v>53</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>11:22</t>
+          <t>11:19</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>117</v>
+        <v>20</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>11:32</t>
+          <t>11:20</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>67</v>
+        <v>21</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3473,21 +3473,21 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:21</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>79</v>
+        <v>116</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>11:50</t>
+          <t>11:22</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>85</v>
+        <v>117</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3528,16 +3528,16 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:32</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>90</v>
+        <v>67</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>12:03</t>
+          <t>11:33</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>98</v>
+        <v>34</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>12:19</t>
+          <t>11:33</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>114</v>
+        <v>34</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,23 +3598,523 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>11:44</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>45</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>11:49</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>50</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>51</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
           <t>10:25:57</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr">
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>85</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>11:51</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>52</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>90</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>11:56</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>57</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>12:03</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>98</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>65</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>12:04</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>65</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>69</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>12:19</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>114</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>10:25:57</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
         <is>
           <t>12:21</t>
         </is>
       </c>
-      <c r="C131" t="inlineStr">
+      <c r="C143" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D131" t="n">
+      <c r="D143" t="n">
         <v>116</v>
       </c>
-      <c r="E131" t="inlineStr">
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>86</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D145" t="n">
+        <v>93</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>95</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>95</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>12:47</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>108</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>12:49</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>110</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>12:51</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>112</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>116</v>
+      </c>
+      <c r="E151" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3631,7 +4131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3644,14 +4144,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:25:57</t>
+          <t>Última actualización: 10:59:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4585,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4099,7 +4599,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>114</v>
+        <v>20</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -4135,23 +4635,73 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>11:33</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>34</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>11:44</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>79</v>
-      </c>
-      <c r="E24" t="inlineStr">
+      <c r="D25" t="n">
+        <v>45</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>95</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4168,7 +4718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4181,14 +4731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:25:57</t>
+          <t>Última actualización: 10:59:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -4714,6 +5264,56 @@
         <v>90</v>
       </c>
       <c r="E25" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>11:56</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>57</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>117</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1586
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E151"/>
+  <dimension ref="A1:E165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:59:30</t>
+          <t>Última actualización: 11:28:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 146</t>
+          <t>Total filas: 160</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2233,11 +2233,11 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>11:32</t>
+          <t>11:28</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>67</v>
+        <v>0</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>11:33</t>
+          <t>11:28</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>11:33</t>
+          <t>11:31</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>34</v>
+        <v>3</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>11:44</t>
+          <t>11:32</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3628,16 +3628,16 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>11:49</t>
+          <t>11:33</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>11:50</t>
+          <t>11:33</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>11:50</t>
+          <t>11:44</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>85</v>
+        <v>16</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>11:51</t>
+          <t>11:46</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,21 +3723,21 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:49</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>90</v>
+        <v>21</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>11:56</t>
+          <t>11:50</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>57</v>
+        <v>85</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>12:03</t>
+          <t>11:50</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>98</v>
+        <v>51</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3803,16 +3803,16 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>11:51</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>65</v>
+        <v>27</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3853,16 +3853,16 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>11:56</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3878,16 +3878,16 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>12:19</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>116</v>
+        <v>35</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3928,16 +3928,16 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>93</v>
+        <v>36</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>95</v>
+        <v>40</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:17</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>95</v>
+        <v>49</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,12 +4023,12 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>12:47</t>
+          <t>12:19</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -4037,7 +4037,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,21 +4048,21 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>12:49</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>12:51</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>112</v>
+        <v>53</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4103,18 +4103,368 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
+          <t>12:25</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>86</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>62</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>64</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>65</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>95</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>12:34</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>95</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>12:47</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>108</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>12:49</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D158" t="n">
+        <v>81</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>12:51</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>83</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>10:59:29</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
           <t>12:55</t>
         </is>
       </c>
-      <c r="C151" t="inlineStr">
+      <c r="C160" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D151" t="n">
+      <c r="D160" t="n">
         <v>116</v>
       </c>
-      <c r="E151" t="inlineStr">
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>13:02</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>94</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>95</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>13:17</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>11X44_P_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>109</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>13:18</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>110</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>116</v>
+      </c>
+      <c r="E165" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4131,7 +4481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4144,14 +4494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:59:30</t>
+          <t>Última actualización: 11:28:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -4610,7 +4960,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4624,7 +4974,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>67</v>
+        <v>4</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4660,7 +5010,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -4674,7 +5024,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -4685,23 +5035,98 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>12:33</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>65</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>10:59:29</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>12:34</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="D27" t="n">
         <v>95</v>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>95</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>13:18</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>110</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4718,7 +5143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4731,14 +5156,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:59:30</t>
+          <t>Última actualización: 11:28:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -5247,7 +5672,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -5261,7 +5686,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>90</v>
+        <v>27</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -5297,25 +5722,100 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>87</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>10:59:29</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>12:56</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D27" t="n">
+      <c r="D28" t="n">
         <v>117</v>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>13:10</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>102</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>13:21</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>113</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1587
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E165"/>
+  <dimension ref="A1:E173"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:28:56</t>
+          <t>Última actualización: 11:53:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 160</t>
+          <t>Total filas: 168</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2233,11 +2233,11 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>85</v>
+        <v>51</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>51</v>
+        <v>85</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3848,7 +3848,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -3862,7 +3862,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>57</v>
+        <v>3</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>12:03</t>
+          <t>12:01</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>98</v>
+        <v>8</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3912,7 +3912,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>12:04</t>
+          <t>12:03</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3962,7 +3962,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>12:04</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>12:17</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>49</v>
+        <v>15</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,12 +4023,12 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>12:19</t>
+          <t>12:17</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -4037,7 +4037,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>114</v>
+        <v>49</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4053,16 +4053,16 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>12:19</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>12:19</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>53</v>
+        <v>26</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>86</v>
+        <v>116</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>64</v>
+        <v>31</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>65</v>
+        <v>86</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>95</v>
+        <v>62</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>12:47</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>108</v>
+        <v>40</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>12:49</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>12:51</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,21 +4323,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>116</v>
+        <v>43</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>13:02</t>
+          <t>12:47</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>94</v>
+        <v>54</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>13:03</t>
+          <t>12:49</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>95</v>
+        <v>56</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>13:17</t>
+          <t>12:51</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>109</v>
+        <v>58</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>13:18</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,23 +4448,223 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
+          <t>11:53:49</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>13:02</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>69</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>11:53:49</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D166" t="n">
+        <v>70</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>11:53:49</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>13:07</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>74</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>11:53:49</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>13:17</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>11X44_P_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>84</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>11:53:49</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>13:18</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>85</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
           <t>11:28:56</t>
         </is>
       </c>
-      <c r="B165" t="inlineStr">
+      <c r="B170" t="inlineStr">
         <is>
           <t>13:24</t>
         </is>
       </c>
-      <c r="C165" t="inlineStr">
+      <c r="C170" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D165" t="n">
+      <c r="D170" t="n">
         <v>116</v>
       </c>
-      <c r="E165" t="inlineStr">
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>11:53:49</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>13:37</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>104</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>11:53:49</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>114</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>11:53:49</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>13:51</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>118</v>
+      </c>
+      <c r="E173" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4481,7 +4681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4494,14 +4694,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:28:56</t>
+          <t>Última actualización: 11:53:49</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -5035,7 +5235,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -5049,7 +5249,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -5085,7 +5285,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5099,7 +5299,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -5110,7 +5310,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5124,9 +5324,34 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>110</v>
+        <v>85</v>
       </c>
       <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>11:53:49</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>13:37</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>104</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5156,7 +5381,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:28:56</t>
+          <t>Última actualización: 11:53:49</t>
         </is>
       </c>
     </row>
@@ -5672,7 +5897,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -5686,7 +5911,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>27</v>
+        <v>2</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -5722,7 +5947,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5736,7 +5961,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>87</v>
+        <v>62</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -5772,7 +5997,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5786,7 +6011,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>102</v>
+        <v>77</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5797,7 +6022,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5811,7 +6036,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>113</v>
+        <v>88</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1588
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E173"/>
+  <dimension ref="A1:E186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:53:49</t>
+          <t>Última actualización: 12:17:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 168</t>
+          <t>Total filas: 181</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2233,11 +2233,11 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>3</v>
+        <v>97</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>97</v>
+        <v>3</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>51</v>
+        <v>85</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>85</v>
+        <v>51</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,12 +4048,12 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>12:19</t>
+          <t>12:17</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -4062,7 +4062,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>114</v>
+        <v>49</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4083,11 +4083,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>26</v>
+        <v>114</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>12:19</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>116</v>
+        <v>2</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>12:24</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>31</v>
+        <v>116</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,12 +4173,12 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>12:25</t>
+          <t>12:24</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>86</v>
+        <v>31</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,21 +4248,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>12:33</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>95</v>
+        <v>39</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>12:34</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>95</v>
+        <v>16</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4328,16 +4328,16 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:33</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>12:47</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>12:49</t>
+          <t>12:34</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>56</v>
+        <v>95</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4403,16 +4403,16 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>12:51</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>116</v>
+        <v>20</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>13:02</t>
+          <t>12:38</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>69</v>
+        <v>21</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>13:03</t>
+          <t>12:47</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>13:07</t>
+          <t>12:49</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>74</v>
+        <v>32</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>13:17</t>
+          <t>12:51</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>84</v>
+        <v>34</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>13:18</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>85</v>
+        <v>116</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:01</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>116</v>
+        <v>44</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4603,16 +4603,16 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>13:37</t>
+          <t>13:02</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4628,16 +4628,16 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>114</v>
+        <v>70</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,23 +4648,348 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
+          <t>12:17:07</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>46</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>12:17:07</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>13:04</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>47</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
           <t>11:53:49</t>
         </is>
       </c>
-      <c r="B173" t="inlineStr">
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>13:07</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>74</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>12:17:07</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>58</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>12:17:07</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>13:17</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>11X44_P_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>60</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>11:53:49</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>13:18</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>85</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>12:17:07</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>13:19</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>62</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>11:28:56</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>116</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>11:53:49</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>13:37</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>104</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>12:17:07</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>81</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>12:17:07</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>90</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>12:17:07</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
         <is>
           <t>13:51</t>
         </is>
       </c>
-      <c r="C173" t="inlineStr">
+      <c r="C184" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D173" t="n">
-        <v>118</v>
-      </c>
-      <c r="E173" t="inlineStr">
+      <c r="D184" t="n">
+        <v>94</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>12:17:07</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>102</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>12:17:07</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>14:03</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>106</v>
+      </c>
+      <c r="E186" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4681,7 +5006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4694,14 +5019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:53:49</t>
+          <t>Última actualización: 12:17:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -5260,7 +5585,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -5274,7 +5599,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>95</v>
+        <v>17</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -5310,21 +5635,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>13:18</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>85</v>
+        <v>47</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5340,18 +5665,93 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
+          <t>13:18</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>85</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>12:17:07</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>13:19</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>62</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>11:53:49</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
           <t>13:37</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D32" t="n">
         <v>104</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>12:17:07</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>81</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5368,7 +5768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5381,14 +5781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:53:49</t>
+          <t>Última actualización: 12:17:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -5972,7 +6372,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5986,7 +6386,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>117</v>
+        <v>39</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -6022,25 +6422,100 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>12:17:07</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>13:11</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>54</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>11:53:49</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>13:21</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D30" t="n">
+      <c r="D31" t="n">
         <v>88</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>12:17:07</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>65</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>12:17:07</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>13:56</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>99</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1589
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E186"/>
+  <dimension ref="A1:E197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:17:07</t>
+          <t>Última actualización: 12:45:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 181</t>
+          <t>Total filas: 192</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>97</v>
+        <v>3</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>3</v>
+        <v>97</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4058,11 +4058,11 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4083,11 +4083,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>114</v>
+        <v>2</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4108,11 +4108,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>2</v>
+        <v>114</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>28</v>
+        <v>116</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>116</v>
+        <v>28</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>12:49</t>
+          <t>12:48</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>12:51</t>
+          <t>12:49</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>34</v>
+        <v>4</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:51</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>116</v>
+        <v>34</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>13:01</t>
+          <t>12:53</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>44</v>
+        <v>8</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>13:02</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>69</v>
+        <v>116</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>13:03</t>
+          <t>13:01</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>70</v>
+        <v>16</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,12 +4648,12 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>13:03</t>
+          <t>13:02</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -4662,7 +4662,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>46</v>
+        <v>69</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>13:04</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>13:07</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>74</v>
+        <v>18</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>13:03</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>13:17</t>
+          <t>13:04</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>11X44_P_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4778,16 +4778,16 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>13:18</t>
+          <t>13:07</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4803,16 +4803,16 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>13:19</t>
+          <t>13:15</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:17</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11X44_P_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>116</v>
+        <v>32</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4853,16 +4853,16 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>13:37</t>
+          <t>13:18</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>13:38</t>
+          <t>13:19</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>81</v>
+        <v>34</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>90</v>
+        <v>36</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4923,21 +4923,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>13:51</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>94</v>
+        <v>116</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>102</v>
+        <v>48</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,23 +4973,298 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
+          <t>12:45:09</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>13:37</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>52</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>11:53:49</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>13:37</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>104</v>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>12:45:09</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>13:38</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>53</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>12:45:09</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>62</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>12:45:09</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>13:51</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>66</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>12:45:09</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>13:59</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>74</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
           <t>12:17:07</t>
         </is>
       </c>
-      <c r="B186" t="inlineStr">
+      <c r="B192" t="inlineStr">
         <is>
           <t>14:03</t>
         </is>
       </c>
-      <c r="C186" t="inlineStr">
+      <c r="C192" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D186" t="n">
+      <c r="D192" t="n">
         <v>106</v>
       </c>
-      <c r="E186" t="inlineStr">
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>12:45:09</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>92</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>12:45:09</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>92</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>12:45:09</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>94</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>12:45:09</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>108</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>12:45:09</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>14:38</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>113</v>
+      </c>
+      <c r="E197" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5006,7 +5281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5019,14 +5294,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:17:07</t>
+          <t>Última actualización: 12:45:09</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -5635,7 +5910,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5649,7 +5924,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>47</v>
+        <v>19</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5685,7 +5960,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5699,7 +5974,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>62</v>
+        <v>34</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -5735,7 +6010,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5749,9 +6024,34 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>81</v>
+        <v>53</v>
       </c>
       <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>12:45:09</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>94</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5781,7 +6081,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:17:07</t>
+          <t>Última actualización: 12:45:09</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6672,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -6386,7 +6686,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -6422,7 +6722,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -6436,7 +6736,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -6472,7 +6772,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -6486,7 +6786,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>65</v>
+        <v>37</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -6497,7 +6797,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -6511,7 +6811,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>99</v>
+        <v>71</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1590
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E197"/>
+  <dimension ref="A1:E205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:45:09</t>
+          <t>Última actualización: 12:59:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 192</t>
+          <t>Total filas: 200</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2233,11 +2233,11 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4662,7 +4662,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>69</v>
+        <v>3</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4687,7 +4687,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4737,7 +4737,7 @@
         </is>
       </c>
       <c r="D176" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4823,7 +4823,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -4837,7 +4837,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,7 +4848,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>85</v>
+        <v>19</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4898,7 +4898,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -4912,7 +4912,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4958,11 +4958,11 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4978,16 +4978,16 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>13:37</t>
+          <t>13:33</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5012,7 +5012,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>104</v>
+        <v>38</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5028,16 +5028,16 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>13:38</t>
+          <t>13:37</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5053,16 +5053,16 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:38</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>13:51</t>
+          <t>13:41</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>66</v>
+        <v>42</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>13:59</t>
+          <t>13:46</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>106</v>
+        <v>62</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>13:51</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>92</v>
+        <v>52</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>13:59</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,21 +5198,21 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>14:19</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>94</v>
+        <v>63</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,21 +5223,21 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,23 +5248,223 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
+          <t>12:59:51</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>77</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>12:59:51</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D198" t="n">
+        <v>78</v>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
           <t>12:45:09</t>
         </is>
       </c>
-      <c r="B197" t="inlineStr">
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>92</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>12:59:51</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>79</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>12:45:09</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>14:19</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>94</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>12:59:51</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>14:32</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D202" t="n">
+        <v>93</v>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>12:45:09</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>108</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>12:59:51</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
         <is>
           <t>14:38</t>
         </is>
       </c>
-      <c r="C197" t="inlineStr">
+      <c r="C204" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D197" t="n">
-        <v>113</v>
-      </c>
-      <c r="E197" t="inlineStr">
+      <c r="D204" t="n">
+        <v>99</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>12:59:51</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>14:51</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>112</v>
+      </c>
+      <c r="E205" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5281,7 +5481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5294,14 +5494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:45:09</t>
+          <t>Última actualización: 12:59:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -5885,7 +6085,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -5899,7 +6099,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>70</v>
+        <v>4</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -5935,7 +6135,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -5949,7 +6149,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>85</v>
+        <v>19</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -5985,7 +6185,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5999,7 +6199,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>104</v>
+        <v>38</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -6035,23 +6235,48 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>12:59:51</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>14:18</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>79</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>12:45:09</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>14:19</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D34" t="n">
+      <c r="D35" t="n">
         <v>94</v>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6068,7 +6293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6081,14 +6306,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:45:09</t>
+          <t>Última actualización: 12:59:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -6697,7 +6922,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -6711,7 +6936,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>77</v>
+        <v>11</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -6747,7 +6972,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -6761,7 +6986,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>88</v>
+        <v>22</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -6797,23 +7022,73 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>12:59:51</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>13:55</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>56</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>12:45:09</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>13:56</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D34" t="n">
         <v>71</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>12:59:51</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>106</v>
+      </c>
+      <c r="E35" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1591
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E205"/>
+  <dimension ref="A1:E213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:59:51</t>
+          <t>Última actualización: 13:33:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 200</t>
+          <t>Total filas: 208</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>3</v>
+        <v>97</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>97</v>
+        <v>3</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4083,11 +4083,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>2</v>
+        <v>114</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4108,11 +4108,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>114</v>
+        <v>2</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>17</v>
+        <v>95</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>95</v>
+        <v>17</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4948,7 +4948,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -4962,7 +4962,7 @@
         </is>
       </c>
       <c r="D185" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,7 +4973,7 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4987,7 +4987,7 @@
         </is>
       </c>
       <c r="D186" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5087,7 +5087,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,7 +5098,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -5112,7 +5112,7 @@
         </is>
       </c>
       <c r="D191" t="n">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5162,7 +5162,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5187,7 +5187,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5212,7 +5212,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>63</v>
+        <v>29</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>77</v>
+        <v>43</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,12 +5273,12 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -5287,7 +5287,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>78</v>
+        <v>43</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,7 +5298,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5308,11 +5308,11 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>14:18</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>79</v>
+        <v>92</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>14:19</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>94</v>
+        <v>44</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:18</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>93</v>
+        <v>45</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5403,16 +5403,16 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:19</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:21</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>99</v>
+        <v>48</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,23 +5448,223 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
+          <t>14:32</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>59</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>12:45:09</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>108</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>13:33:52</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>14:38</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>65</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>13:33:52</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
           <t>14:51</t>
         </is>
       </c>
-      <c r="C205" t="inlineStr">
+      <c r="C208" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D205" t="n">
-        <v>112</v>
-      </c>
-      <c r="E205" t="inlineStr">
+      <c r="D208" t="n">
+        <v>78</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>13:33:52</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D209" t="n">
+        <v>86</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>13:33:52</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>86</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>13:33:52</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>15:06</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>93</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>13:33:52</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>105</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>13:33:52</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>110</v>
+      </c>
+      <c r="E213" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5481,7 +5681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5494,14 +5694,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:59:51</t>
+          <t>Última actualización: 13:33:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -6185,7 +6385,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -6199,7 +6399,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -6235,7 +6435,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -6249,7 +6449,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>79</v>
+        <v>45</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -6277,6 +6477,56 @@
         <v>94</v>
       </c>
       <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>13:33:52</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>86</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>13:33:52</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>105</v>
+      </c>
+      <c r="E37" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6293,7 +6543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6306,14 +6556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:59:51</t>
+          <t>Última actualización: 13:33:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -7022,7 +7272,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7036,7 +7286,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -7072,7 +7322,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7086,11 +7336,36 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>106</v>
+        <v>72</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>13:33:52</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>92</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1592
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E213"/>
+  <dimension ref="A1:E226"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:33:52</t>
+          <t>Última actualización: 14:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 208</t>
+          <t>Total filas: 221</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>97</v>
+        <v>3</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>3</v>
+        <v>97</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>85</v>
+        <v>51</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>51</v>
+        <v>85</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4058,11 +4058,11 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4083,11 +4083,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>114</v>
+        <v>2</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4108,11 +4108,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>2</v>
+        <v>114</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>116</v>
+        <v>28</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>28</v>
+        <v>116</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>95</v>
+        <v>17</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>17</v>
+        <v>95</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -5198,21 +5198,21 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>14:02</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,12 +5223,12 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>14:03</t>
+          <t>14:02</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -5237,7 +5237,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>106</v>
+        <v>2</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,21 +5248,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:03</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>43</v>
+        <v>106</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:04</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>43</v>
+        <v>4</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,12 +5298,12 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -5312,7 +5312,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>78</v>
+        <v>43</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,12 +5323,12 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -5337,7 +5337,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>92</v>
+        <v>43</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>14:18</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>14:19</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>94</v>
+        <v>17</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>14:21</t>
+          <t>14:18</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>14:32</t>
+          <t>14:19</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>59</v>
+        <v>19</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,21 +5473,21 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>14:33</t>
+          <t>14:21</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>108</v>
+        <v>21</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5503,16 +5503,16 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:32</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>78</v>
+        <v>33</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>86</v>
+        <v>47</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>14:51</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>93</v>
+        <v>51</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>105</v>
+        <v>59</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5653,18 +5653,343 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
+          <t>14:59</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>86</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>60</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>13:33:52</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>15:06</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>93</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>67</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>13:33:52</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D217" t="n">
+        <v>105</v>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>15:19</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>79</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>13:33:52</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
           <t>15:23</t>
         </is>
       </c>
-      <c r="C213" t="inlineStr">
+      <c r="C219" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D213" t="n">
+      <c r="D219" t="n">
         <v>110</v>
       </c>
-      <c r="E213" t="inlineStr">
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>15:24</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>84</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>15:38</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>98</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>101</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>15:48</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>108</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>15:51</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>111</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>114</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>117</v>
+      </c>
+      <c r="E226" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5681,7 +6006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5694,14 +6019,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:33:52</t>
+          <t>Última actualización: 14:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -6460,7 +6785,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -6474,7 +6799,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6510,23 +6835,73 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>60</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>13:33:52</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B38" t="inlineStr">
         <is>
           <t>15:18</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D37" t="n">
+      <c r="D38" t="n">
         <v>105</v>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>15:19</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>79</v>
+      </c>
+      <c r="E39" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6543,7 +6918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6556,14 +6931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:33:52</t>
+          <t>Última actualización: 14:00:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -7347,25 +7722,100 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>14:46</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>46</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>13:33:52</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>15:05</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D36" t="n">
+      <c r="D37" t="n">
         <v>92</v>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>15:09</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>69</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>15:46</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>106</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1593
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E226"/>
+  <dimension ref="A1:E237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:00:00</t>
+          <t>Última actualización: 14:27:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 221</t>
+          <t>Total filas: 232</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2958,7 +2958,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4083,11 +4083,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>2</v>
+        <v>114</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4108,11 +4108,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>114</v>
+        <v>2</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5408,11 +5408,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5512,7 +5512,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>59</v>
+        <v>5</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>14:38</t>
+          <t>14:33</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>38</v>
+        <v>6</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,21 +5573,21 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:38</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>47</v>
+        <v>11</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5598,21 +5598,21 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>51</v>
+        <v>14</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5628,16 +5628,16 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>59</v>
+        <v>47</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:51</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>86</v>
+        <v>24</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>93</v>
+        <v>32</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5728,16 +5728,16 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5753,16 +5753,16 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>105</v>
+        <v>93</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5778,16 +5778,16 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>15:19</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>110</v>
+        <v>44</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:14</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>84</v>
+        <v>47</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>98</v>
+        <v>51</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5878,16 +5878,16 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:19</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,12 +5898,12 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -5912,7 +5912,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>108</v>
+        <v>56</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5928,16 +5928,16 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>111</v>
+        <v>84</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>114</v>
+        <v>68</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,23 +5973,298 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
+          <t>14:27:41</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>15:37</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>70</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>14:27:41</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>15:38</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D227" t="n">
+        <v>71</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>14:27:41</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>15:41</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>74</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>14:27:41</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>80</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
           <t>14:00:00</t>
         </is>
       </c>
-      <c r="B226" t="inlineStr">
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>15:48</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>108</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>14:27:41</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>15:51</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>84</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>14:27:41</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>87</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
         <is>
           <t>15:57</t>
         </is>
       </c>
-      <c r="C226" t="inlineStr">
+      <c r="C233" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D226" t="n">
+      <c r="D233" t="n">
         <v>117</v>
       </c>
-      <c r="E226" t="inlineStr">
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>14:27:41</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>15:58</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>91</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>14:27:41</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>16:09</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>102</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>14:27:41</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>16:11</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>104</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>14:27:41</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>116</v>
+      </c>
+      <c r="E237" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6006,7 +6281,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6019,14 +6294,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:00:00</t>
+          <t>Última actualización: 14:27:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -6810,7 +7085,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -6824,7 +7099,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>86</v>
+        <v>32</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -6860,7 +7135,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6874,7 +7149,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>105</v>
+        <v>51</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -6902,6 +7177,31 @@
         <v>79</v>
       </c>
       <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>14:27:41</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>116</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6918,7 +7218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6931,14 +7231,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:00:00</t>
+          <t>Última actualización: 14:27:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -7697,7 +7997,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -7711,7 +8011,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>72</v>
+        <v>18</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -7797,23 +8097,73 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>14:27:41</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>15:13</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>46</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>14:27:41</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>78</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>14:00:00</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>15:46</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D39" t="n">
+      <c r="D41" t="n">
         <v>106</v>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1594
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E237"/>
+  <dimension ref="A1:E245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:27:41</t>
+          <t>Última actualización: 14:50:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 232</t>
+          <t>Total filas: 240</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4058,11 +4058,11 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>28</v>
+        <v>116</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>116</v>
+        <v>28</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -5358,7 +5358,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -5383,7 +5383,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5648,21 +5648,21 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>14:51</t>
+          <t>14:50</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:51</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,12 +5698,12 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:53</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -5712,7 +5712,7 @@
         </is>
       </c>
       <c r="D215" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,12 +5723,12 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -5737,7 +5737,7 @@
         </is>
       </c>
       <c r="D216" t="n">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,21 +5748,21 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>15:06</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>93</v>
+        <v>9</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5778,16 +5778,16 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,21 +5798,21 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D219" t="n">
-        <v>44</v>
+        <v>11</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,21 +5823,21 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>15:14</t>
+          <t>15:03</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,21 +5848,21 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>51</v>
+        <v>93</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5878,16 +5878,16 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>15:19</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>56</v>
+        <v>21</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:14</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>84</v>
+        <v>47</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5953,16 +5953,16 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>68</v>
+        <v>51</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>15:37</t>
+          <t>15:19</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>70</v>
+        <v>29</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,21 +6023,21 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>74</v>
+        <v>84</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:37</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>108</v>
+        <v>47</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:38</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>84</v>
+        <v>48</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>87</v>
+        <v>51</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>117</v>
+        <v>57</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>15:58</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>102</v>
+        <v>61</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>16:11</t>
+          <t>15:54</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>104</v>
+        <v>64</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,23 +6248,223 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
+          <t>14:50:32</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>66</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>14:00:00</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>117</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
           <t>14:27:41</t>
         </is>
       </c>
-      <c r="B237" t="inlineStr">
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>15:58</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D239" t="n">
+        <v>91</v>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>14:50:32</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>16:09</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>79</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>14:50:32</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>16:11</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>81</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>14:27:41</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
         <is>
           <t>16:23</t>
         </is>
       </c>
-      <c r="C237" t="inlineStr">
+      <c r="C242" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D237" t="n">
+      <c r="D242" t="n">
         <v>116</v>
       </c>
-      <c r="E237" t="inlineStr">
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>14:50:32</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>94</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>14:50:32</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>105</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>14:50:32</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>16:47</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>117</v>
+      </c>
+      <c r="E245" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6281,7 +6481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6294,14 +6494,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:27:41</t>
+          <t>Última actualización: 14:50:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -7085,12 +7285,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>14:59</t>
+          <t>14:53</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -7099,7 +7299,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>32</v>
+        <v>3</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -7110,12 +7310,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:59</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -7124,7 +7324,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -7135,21 +7335,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>51</v>
+        <v>60</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -7160,12 +7360,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>15:19</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -7174,7 +7374,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>79</v>
+        <v>51</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -7185,23 +7385,73 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>14:50:32</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>15:19</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>29</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>14:27:41</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>16:23</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D40" t="n">
+      <c r="D41" t="n">
         <v>116</v>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>14:50:32</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>94</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7218,7 +7468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7231,14 +7481,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:27:41</t>
+          <t>Última actualización: 14:50:32</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -8122,50 +8372,100 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:17</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>78</v>
+        <v>27</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>78</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>14:50:32</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>15:46</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D41" t="n">
-        <v>106</v>
-      </c>
-      <c r="E41" t="inlineStr">
+      <c r="D42" t="n">
+        <v>56</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>14:50:32</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>16:43</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>113</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1595
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E245"/>
+  <dimension ref="A1:E255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:50:32</t>
+          <t>Última actualización: 15:21:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 240</t>
+          <t>Total filas: 250</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>3</v>
+        <v>97</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>97</v>
+        <v>3</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4058,11 +4058,11 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4083,11 +4083,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>114</v>
+        <v>2</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4108,11 +4108,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>2</v>
+        <v>114</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>116</v>
+        <v>28</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>28</v>
+        <v>116</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4733,7 +4733,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5358,7 +5358,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -5383,7 +5383,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>15:21:39</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:21</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,12 +6023,12 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>15:21:39</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>15:24</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -6037,7 +6037,7 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>84</v>
+        <v>2</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>15:35</t>
+          <t>15:24</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>45</v>
+        <v>84</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,12 +6073,12 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>15:21:39</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>15:37</t>
+          <t>15:34</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -6087,7 +6087,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>47</v>
+        <v>13</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>15:21:39</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>15:38</t>
+          <t>15:35</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>48</v>
+        <v>14</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6128,16 +6128,16 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:37</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>15:21:39</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:38</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>15:21:39</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>108</v>
+        <v>20</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>15:21:39</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>15:51</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,21 +6223,21 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>15:54</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>64</v>
+        <v>108</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>15:21:39</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:51</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>66</v>
+        <v>30</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>15:21:39</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:54</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>117</v>
+        <v>33</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,12 +6298,12 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>15:21:39</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>15:58</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -6312,7 +6312,7 @@
         </is>
       </c>
       <c r="D239" t="n">
-        <v>91</v>
+        <v>35</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>79</v>
+        <v>117</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>16:11</t>
+          <t>15:58</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>15:21:39</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>15:59</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>116</v>
+        <v>38</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>15:21:39</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:09</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>94</v>
+        <v>48</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,21 +6423,21 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>15:21:39</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:11</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>105</v>
+        <v>50</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,23 +6448,273 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
+          <t>15:21:39</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>62</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>15:21:39</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>62</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
           <t>14:50:32</t>
         </is>
       </c>
-      <c r="B245" t="inlineStr">
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>16:24</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>94</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>15:21:39</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D248" t="n">
+        <v>74</v>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>15:21:39</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>74</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>15:21:39</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>16:46</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>85</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>15:21:39</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
         <is>
           <t>16:47</t>
         </is>
       </c>
-      <c r="C245" t="inlineStr">
+      <c r="C251" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D245" t="n">
-        <v>117</v>
-      </c>
-      <c r="E245" t="inlineStr">
+      <c r="D251" t="n">
+        <v>86</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>15:21:39</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>90</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>15:21:39</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>98</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>15:21:39</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D254" t="n">
+        <v>98</v>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>15:21:39</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>17:11</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>110</v>
+      </c>
+      <c r="E255" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6481,7 +6731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6494,14 +6744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:50:32</t>
+          <t>Última actualización: 15:21:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -7410,7 +7660,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>15:21:39</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7424,7 +7674,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>116</v>
+        <v>62</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -7452,6 +7702,31 @@
         <v>94</v>
       </c>
       <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>15:21:39</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>98</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7468,7 +7743,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7481,14 +7756,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:50:32</t>
+          <t>Última actualización: 15:21:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -8397,37 +8672,37 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>15:21:39</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>78</v>
+        <v>2</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>15:46</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -8436,7 +8711,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>56</v>
+        <v>78</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -8447,25 +8722,100 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
+          <t>15:21:39</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>15:46</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>25</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>15:21:39</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>16:42</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>81</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>14:50:32</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>16:43</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D43" t="n">
+      <c r="D45" t="n">
         <v>113</v>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>15:21:39</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>94</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1596
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E255"/>
+  <dimension ref="A1:E270"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:21:39</t>
+          <t>Última actualización: 16:00:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 250</t>
+          <t>Total filas: 265</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>97</v>
+        <v>3</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>3</v>
+        <v>97</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>51</v>
+        <v>85</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>85</v>
+        <v>51</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>28</v>
+        <v>116</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>116</v>
+        <v>28</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>17</v>
+        <v>95</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>95</v>
+        <v>17</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5408,11 +5408,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6398,21 +6398,21 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>15:21:39</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>16:09</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,21 +6423,21 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>15:21:39</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>16:11</t>
+          <t>16:03</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>50</v>
+        <v>3</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>15:21:39</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:09</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>62</v>
+        <v>9</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,21 +6473,21 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>15:21:39</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:11</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>62</v>
+        <v>11</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6498,21 +6498,21 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>16:24</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>94</v>
+        <v>23</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,21 +6523,21 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>15:21:39</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>74</v>
+        <v>23</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,21 +6548,21 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>15:21:39</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>16:35</t>
+          <t>16:24</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>15:21:39</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>16:46</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>85</v>
+        <v>35</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,21 +6598,21 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>15:21:39</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:35</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>86</v>
+        <v>35</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,21 +6623,21 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>15:21:39</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:43</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>90</v>
+        <v>43</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6653,16 +6653,16 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:46</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,21 +6673,21 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>15:21:39</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:47</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>98</v>
+        <v>47</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,23 +6698,398 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>15:21:39</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
+          <t>16:48</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>48</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>51</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>59</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>16:59</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>59</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
           <t>17:11</t>
         </is>
       </c>
-      <c r="C255" t="inlineStr">
+      <c r="C259" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D255" t="n">
-        <v>110</v>
-      </c>
-      <c r="E255" t="inlineStr">
+      <c r="D259" t="n">
+        <v>71</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>17:21</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>81</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>17:23</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>83</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D262" t="n">
+        <v>95</v>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D263" t="n">
+        <v>95</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D264" t="n">
+        <v>96</v>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>17:41</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>101</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>107</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>107</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>17:51</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>111</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>119</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>119</v>
+      </c>
+      <c r="E270" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6731,7 +7106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6744,14 +7119,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:21:39</t>
+          <t>Última actualización: 16:00:50</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -7660,7 +8035,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>15:21:39</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7674,7 +8049,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>62</v>
+        <v>23</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -7710,7 +8085,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>15:21:39</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7724,9 +8099,59 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>98</v>
+        <v>59</v>
       </c>
       <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>107</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>107</v>
+      </c>
+      <c r="E45" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7756,7 +8181,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:21:39</t>
+          <t>Última actualización: 16:00:50</t>
         </is>
       </c>
     </row>
@@ -8747,7 +9172,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>15:21:39</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8761,7 +9186,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -8797,7 +9222,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>15:21:39</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8811,7 +9236,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>94</v>
+        <v>55</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1597
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E270"/>
+  <dimension ref="A1:E284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:00:50</t>
+          <t>Última actualización: 16:36:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 265</t>
+          <t>Total filas: 279</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2233,11 +2233,11 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4058,11 +4058,11 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5383,7 +5383,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5408,11 +5408,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -6623,21 +6623,21 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:36:16</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>16:43</t>
+          <t>16:36</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,21 +6648,21 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>15:21:39</t>
+          <t>16:36:16</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>16:46</t>
+          <t>16:40</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>85</v>
+        <v>4</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6678,16 +6678,16 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>16:47</t>
+          <t>16:43</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,21 +6698,21 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>15:21:39</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>16:48</t>
+          <t>16:46</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>48</v>
+        <v>85</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,21 +6723,21 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:36:16</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>16:51</t>
+          <t>16:47</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>51</v>
+        <v>11</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,21 +6748,21 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:36:16</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:48</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>59</v>
+        <v>12</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,21 +6773,21 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:36:16</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:51</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6803,16 +6803,16 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>17:11</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6828,16 +6828,16 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>81</v>
+        <v>59</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,21 +6848,21 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:36:16</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>17:23</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>83</v>
+        <v>24</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,21 +6873,21 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:36:16</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>95</v>
+        <v>24</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,21 +6898,21 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:36:16</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>95</v>
+        <v>28</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6928,16 +6928,16 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:11</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>96</v>
+        <v>71</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,21 +6948,21 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:36:16</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:12</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>101</v>
+        <v>36</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,21 +6973,21 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:36:16</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>107</v>
+        <v>45</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -7003,16 +7003,16 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:23</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>107</v>
+        <v>83</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,21 +7023,21 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:36:16</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>111</v>
+        <v>48</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,21 +7048,21 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:36:16</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>119</v>
+        <v>59</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,23 +7073,373 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
+          <t>16:36:16</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>59</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
           <t>16:00:50</t>
         </is>
       </c>
-      <c r="B270" t="inlineStr">
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>17:36</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>96</v>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>16:36:16</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>17:37</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D272" t="n">
+        <v>61</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>16:36:16</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>17:39</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>63</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>16:36:16</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>17:41</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>65</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D275" t="n">
+        <v>107</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>107</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>16:36:16</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>72</v>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>16:36:16</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>72</v>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>16:36:16</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>17:51</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>75</v>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>16:36:16</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
         <is>
           <t>17:59</t>
         </is>
       </c>
-      <c r="C270" t="inlineStr">
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>83</v>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D270" t="n">
+      <c r="D281" t="n">
         <v>119</v>
       </c>
-      <c r="E270" t="inlineStr">
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>16:36:16</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>84</v>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>16:36:16</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>18:12</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>96</v>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>16:36:16</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>108</v>
+      </c>
+      <c r="E284" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7106,7 +7456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7119,14 +7469,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:00:50</t>
+          <t>Última actualización: 16:36:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -8110,21 +8460,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:36:16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>107</v>
+        <v>24</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -8145,13 +8495,88 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D45" t="n">
         <v>107</v>
       </c>
       <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>16:00:50</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>107</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>16:36:16</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>72</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>16:36:16</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>72</v>
+      </c>
+      <c r="E48" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8168,7 +8593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8181,14 +8606,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:00:50</t>
+          <t>Última actualización: 16:36:16</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 44</t>
         </is>
       </c>
     </row>
@@ -9172,12 +9597,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:36:16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>16:42</t>
+          <t>16:39</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -9186,7 +9611,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>42</v>
+        <v>3</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -9197,12 +9622,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>16:43</t>
+          <t>16:42</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -9211,7 +9636,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>113</v>
+        <v>42</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -9222,23 +9647,98 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
+          <t>14:50:32</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>16:43</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>113</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
           <t>16:00:50</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>16:55</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D46" t="n">
+      <c r="D47" t="n">
         <v>55</v>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>16:36:16</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>20</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>16:36:16</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>18:26</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>110</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1598
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E284"/>
+  <dimension ref="A1:E292"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:36:16</t>
+          <t>Última actualización: 16:52:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 279</t>
+          <t>Total filas: 287</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>85</v>
+        <v>51</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>51</v>
+        <v>85</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>116</v>
+        <v>28</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>28</v>
+        <v>116</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5408,11 +5408,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -6798,21 +6798,21 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>16:59</t>
+          <t>16:52</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6833,7 +6833,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -6848,21 +6848,21 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>17:00</t>
+          <t>16:59</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>24</v>
+        <v>59</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6887,7 +6887,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,21 +6898,21 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>17:04</t>
+          <t>17:00</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D263" t="n">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,21 +6923,21 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>17:11</t>
+          <t>17:03</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>71</v>
+        <v>11</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6953,16 +6953,16 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>17:12</t>
+          <t>17:04</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,21 +6973,21 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>17:21</t>
+          <t>17:11</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -7003,16 +7003,16 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>17:23</t>
+          <t>17:11</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,21 +7023,21 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>17:24</t>
+          <t>17:12</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,21 +7048,21 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:21</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>59</v>
+        <v>29</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,21 +7073,21 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:23</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,21 +7098,21 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:24</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>96</v>
+        <v>32</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,21 +7123,21 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,21 +7148,21 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>17:39</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>63</v>
+        <v>43</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,21 +7173,21 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>65</v>
+        <v>96</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,21 +7198,21 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>107</v>
+        <v>45</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,21 +7223,21 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:36:16</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:39</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>107</v>
+        <v>63</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,21 +7248,21 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>17:48</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,21 +7273,21 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>17:48</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>72</v>
+        <v>49</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,21 +7298,21 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>75</v>
+        <v>107</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,21 +7323,21 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,21 +7348,21 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:48</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>119</v>
+        <v>56</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,21 +7373,21 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:48</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,21 +7398,21 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>17:51</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>96</v>
+        <v>59</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,23 +7423,223 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>119</v>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>16:52:15</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>17:59</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>67</v>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>16:52:15</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>68</v>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>16:52:15</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>18:12</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>80</v>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>16:52:15</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>18:12</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>80</v>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>16:52:15</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>91</v>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>16:52:15</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
           <t>18:24</t>
         </is>
       </c>
-      <c r="C284" t="inlineStr">
+      <c r="C290" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D284" t="n">
-        <v>108</v>
-      </c>
-      <c r="E284" t="inlineStr">
+      <c r="D290" t="n">
+        <v>92</v>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>16:52:15</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>103</v>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>16:52:15</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>18:39</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>107</v>
+      </c>
+      <c r="E292" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7469,7 +7669,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:36:16</t>
+          <t>Última actualización: 16:52:15</t>
         </is>
       </c>
     </row>
@@ -8460,7 +8660,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -8474,7 +8674,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -8495,7 +8695,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -8520,7 +8720,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -8535,7 +8735,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8549,7 +8749,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -8560,7 +8760,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -8574,7 +8774,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -8593,7 +8793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8606,14 +8806,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:36:16</t>
+          <t>Última actualización: 16:52:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 44</t>
+          <t>Total filas: 45</t>
         </is>
       </c>
     </row>
@@ -9672,12 +9872,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:54</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -9686,7 +9886,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>55</v>
+        <v>2</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -9697,12 +9897,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -9711,7 +9911,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -9727,18 +9927,43 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>20</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>16:52:15</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
           <t>18:26</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D49" t="n">
-        <v>110</v>
-      </c>
-      <c r="E49" t="inlineStr">
+      <c r="D50" t="n">
+        <v>94</v>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1599
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E292"/>
+  <dimension ref="A1:E301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:52:15</t>
+          <t>Última actualización: 17:15:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 287</t>
+          <t>Total filas: 296</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4083,11 +4083,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>2</v>
+        <v>114</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4108,11 +4108,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>114</v>
+        <v>2</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -7048,7 +7048,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
@@ -7062,7 +7062,7 @@
         </is>
       </c>
       <c r="D269" t="n">
-        <v>29</v>
+        <v>6</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,7 +7073,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -7087,7 +7087,7 @@
         </is>
       </c>
       <c r="D270" t="n">
-        <v>83</v>
+        <v>8</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7123,21 +7123,21 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>17:35</t>
+          <t>17:33</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>43</v>
+        <v>18</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,7 +7148,7 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
@@ -7162,7 +7162,7 @@
         </is>
       </c>
       <c r="D273" t="n">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,21 +7173,21 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>96</v>
+        <v>20</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,12 +7198,12 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -7212,7 +7212,7 @@
         </is>
       </c>
       <c r="D275" t="n">
-        <v>45</v>
+        <v>21</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,21 +7223,21 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>16:36:16</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>17:39</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>63</v>
+        <v>45</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,12 +7248,12 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>16:36:16</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>17:40</t>
+          <t>17:39</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
@@ -7262,7 +7262,7 @@
         </is>
       </c>
       <c r="D277" t="n">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7278,16 +7278,16 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:40</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,21 +7298,21 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>17:47</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>107</v>
+        <v>26</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7348,21 +7348,21 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>17:48</t>
+          <t>17:47</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,7 +7373,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -7383,11 +7383,11 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7403,16 +7403,16 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>17:51</t>
+          <t>17:48</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,21 +7423,21 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>17:59</t>
+          <t>17:51</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>119</v>
+        <v>36</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,7 +7448,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -7462,7 +7462,7 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,12 +7473,12 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>17:59</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -7487,7 +7487,7 @@
         </is>
       </c>
       <c r="D286" t="n">
-        <v>68</v>
+        <v>119</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,21 +7498,21 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>80</v>
+        <v>45</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,12 +7523,12 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>18:11</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -7537,7 +7537,7 @@
         </is>
       </c>
       <c r="D288" t="n">
-        <v>80</v>
+        <v>56</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,21 +7548,21 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>91</v>
+        <v>57</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>92</v>
+        <v>57</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7603,16 +7603,16 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>103</v>
+        <v>80</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7623,23 +7623,248 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
+          <t>17:15:35</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>68</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>17:15:35</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>69</v>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>17:15:35</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>80</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>17:15:35</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>18:38</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>83</v>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
           <t>16:52:15</t>
         </is>
       </c>
-      <c r="B292" t="inlineStr">
+      <c r="B296" t="inlineStr">
         <is>
           <t>18:39</t>
         </is>
       </c>
-      <c r="C292" t="inlineStr">
+      <c r="C296" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D292" t="n">
+      <c r="D296" t="n">
         <v>107</v>
       </c>
-      <c r="E292" t="inlineStr">
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>17:15:35</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>18:51</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>96</v>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>17:15:35</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>98</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>17:15:35</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>105</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>17:15:35</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>113</v>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>17:15:35</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>19:12</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>117</v>
+      </c>
+      <c r="E301" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7669,7 +7894,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:52:15</t>
+          <t>Última actualización: 17:15:35</t>
         </is>
       </c>
     </row>
@@ -8695,7 +8920,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -8710,7 +8935,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8720,11 +8945,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>107</v>
+        <v>32</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -8745,7 +8970,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -8760,7 +8985,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -8770,11 +8995,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>56</v>
+        <v>33</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -8793,7 +9018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8806,14 +9031,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:52:15</t>
+          <t>Última actualización: 17:15:35</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 45</t>
+          <t>Total filas: 46</t>
         </is>
       </c>
     </row>
@@ -9947,23 +10172,48 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
+          <t>17:15:35</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>18:25</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>70</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>16:52:15</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B51" t="inlineStr">
         <is>
           <t>18:26</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D50" t="n">
+      <c r="D51" t="n">
         <v>94</v>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1600
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E301"/>
+  <dimension ref="A1:E310"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:15:35</t>
+          <t>Última actualización: 17:46:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 296</t>
+          <t>Total filas: 305</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>28</v>
+        <v>116</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>116</v>
+        <v>28</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>95</v>
+        <v>17</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>17</v>
+        <v>95</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -6883,7 +6883,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D262" t="n">
@@ -6908,7 +6908,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D263" t="n">
@@ -6973,7 +6973,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -6983,11 +6983,11 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>19</v>
+        <v>71</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,7 +6998,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -7008,11 +7008,11 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>71</v>
+        <v>19</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7323,7 +7323,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -7333,11 +7333,11 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>107</v>
+        <v>1</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,7 +7348,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>32</v>
+        <v>107</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,7 +7373,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -7383,11 +7383,11 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,7 +7398,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -7408,11 +7408,11 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,7 +7423,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
@@ -7437,7 +7437,7 @@
         </is>
       </c>
       <c r="D284" t="n">
-        <v>36</v>
+        <v>5</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,7 +7448,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -7462,7 +7462,7 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7498,7 +7498,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
@@ -7512,7 +7512,7 @@
         </is>
       </c>
       <c r="D287" t="n">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,21 +7523,21 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>18:11</t>
+          <t>18:01</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>56</v>
+        <v>15</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,21 +7548,21 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>18:03</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>18:11</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,7 +7598,7 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
@@ -7608,11 +7608,11 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7623,21 +7623,21 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,12 +7648,12 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
@@ -7662,7 +7662,7 @@
         </is>
       </c>
       <c r="D293" t="n">
-        <v>69</v>
+        <v>26</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,21 +7673,21 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>80</v>
+        <v>37</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,21 +7698,21 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>18:38</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>83</v>
+        <v>38</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,21 +7723,21 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>18:39</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>107</v>
+        <v>49</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,21 +7748,21 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>18:51</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>96</v>
+        <v>50</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,21 +7773,21 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:38</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>98</v>
+        <v>52</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7798,21 +7798,21 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:39</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,21 +7823,21 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:41</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>113</v>
+        <v>55</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,23 +7848,248 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
+          <t>18:51</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>65</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>17:46:20</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>67</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>17:46:20</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>74</v>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>17:46:20</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>82</v>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>17:46:20</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
           <t>19:12</t>
         </is>
       </c>
-      <c r="C301" t="inlineStr">
+      <c r="C305" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D301" t="n">
-        <v>117</v>
-      </c>
-      <c r="E301" t="inlineStr">
+      <c r="D305" t="n">
+        <v>86</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>17:46:20</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>19:19</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>93</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>17:46:20</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>97</v>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>17:46:20</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D308" t="n">
+        <v>98</v>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>17:46:20</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>110</v>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>17:46:20</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D310" t="n">
+        <v>114</v>
+      </c>
+      <c r="E310" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7881,7 +8106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7894,14 +8119,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:15:35</t>
+          <t>Última actualización: 17:46:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 45</t>
         </is>
       </c>
     </row>
@@ -8910,7 +9135,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -8920,11 +9145,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>107</v>
+        <v>1</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -8935,7 +9160,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -8945,11 +9170,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>32</v>
+        <v>107</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -8985,7 +9210,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -8999,9 +9224,59 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>17:46:20</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>98</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>17:46:20</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>110</v>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9018,7 +9293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9031,14 +9306,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:15:35</t>
+          <t>Última actualización: 17:46:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 46</t>
+          <t>Total filas: 47</t>
         </is>
       </c>
     </row>
@@ -10197,7 +10472,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -10211,11 +10486,36 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>94</v>
+        <v>40</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>17:46:20</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>92</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1601
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E310"/>
+  <dimension ref="A1:E319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:46:20</t>
+          <t>Última actualización: 18:02:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 305</t>
+          <t>Total filas: 314</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2958,7 +2958,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D105" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4058,11 +4058,11 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4083,11 +4083,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>114</v>
+        <v>2</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4108,11 +4108,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>2</v>
+        <v>114</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>116</v>
+        <v>28</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>28</v>
+        <v>116</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>18:11</t>
+          <t>18:04</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,21 +7598,21 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>18:12</t>
+          <t>18:11</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>57</v>
+        <v>9</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7623,7 +7623,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -7633,11 +7633,11 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>80</v>
+        <v>26</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,21 +7673,21 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:12</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>37</v>
+        <v>80</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,21 +7698,21 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,21 +7723,21 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>49</v>
+        <v>22</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,12 +7748,12 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>18:36</t>
+          <t>18:33</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
@@ -7762,7 +7762,7 @@
         </is>
       </c>
       <c r="D297" t="n">
-        <v>50</v>
+        <v>31</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,21 +7773,21 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>18:38</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7798,21 +7798,21 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>18:39</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>107</v>
+        <v>50</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,21 +7823,21 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>18:41</t>
+          <t>18:38</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,21 +7848,21 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>18:51</t>
+          <t>18:39</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>65</v>
+        <v>107</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -7873,21 +7873,21 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:41</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -7898,21 +7898,21 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:48</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>74</v>
+        <v>46</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -7923,21 +7923,21 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>82</v>
+        <v>49</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -7948,21 +7948,21 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,21 +7973,21 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -7998,21 +7998,21 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:01</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>97</v>
+        <v>59</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,21 +8023,21 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>98</v>
+        <v>66</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,21 +8048,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>110</v>
+        <v>70</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8073,23 +8073,248 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
+          <t>18:02:23</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D310" t="n">
+        <v>75</v>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
           <t>17:46:20</t>
         </is>
       </c>
-      <c r="B310" t="inlineStr">
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>19:19</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D311" t="n">
+        <v>93</v>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>18:02:23</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>81</v>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>18:02:23</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>19:24</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D313" t="n">
+        <v>82</v>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>18:02:23</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D314" t="n">
+        <v>94</v>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>18:02:23</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
         <is>
           <t>19:40</t>
         </is>
       </c>
-      <c r="C310" t="inlineStr">
+      <c r="C315" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D310" t="n">
-        <v>114</v>
-      </c>
-      <c r="E310" t="inlineStr">
+      <c r="D315" t="n">
+        <v>98</v>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>18:02:23</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D316" t="n">
+        <v>105</v>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>18:02:23</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>19:53</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D317" t="n">
+        <v>111</v>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>18:02:23</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>19:55</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D318" t="n">
+        <v>113</v>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>18:02:23</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D319" t="n">
+        <v>118</v>
+      </c>
+      <c r="E319" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8119,7 +8344,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:46:20</t>
+          <t>Última actualización: 18:02:24</t>
         </is>
       </c>
     </row>
@@ -9235,7 +9460,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -9249,7 +9474,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -9260,7 +9485,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -9274,7 +9499,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>110</v>
+        <v>94</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -9306,7 +9531,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:46:20</t>
+          <t>Última actualización: 18:02:24</t>
         </is>
       </c>
     </row>
@@ -10472,7 +10697,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -10486,7 +10711,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -10497,7 +10722,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -10511,7 +10736,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1602
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E319"/>
+  <dimension ref="A1:E328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:02:24</t>
+          <t>Última actualización: 18:36:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 314</t>
+          <t>Total filas: 323</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>3</v>
+        <v>97</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>97</v>
+        <v>3</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4058,11 +4058,11 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>28</v>
+        <v>116</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>116</v>
+        <v>28</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>17</v>
+        <v>95</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>95</v>
+        <v>17</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5383,7 +5383,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5408,11 +5408,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6973,7 +6973,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -6983,11 +6983,11 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>71</v>
+        <v>19</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,7 +6998,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -7008,11 +7008,11 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>19</v>
+        <v>71</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7623,7 +7623,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -7633,11 +7633,11 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7798,7 +7798,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
@@ -7808,11 +7808,11 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,21 +7823,21 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>18:38</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>36</v>
+        <v>50</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,21 +7848,21 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>18:39</t>
+          <t>18:36</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>107</v>
+        <v>0</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -7878,16 +7878,16 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>18:41</t>
+          <t>18:38</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -7898,21 +7898,21 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>18:48</t>
+          <t>18:39</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>46</v>
+        <v>107</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -7923,21 +7923,21 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>18:51</t>
+          <t>18:41</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -7948,21 +7948,21 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:48</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,21 +7973,21 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>19:00</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>58</v>
+        <v>15</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -7998,21 +7998,21 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>19:01</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>59</v>
+        <v>17</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,21 +8023,21 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:00</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,21 +8048,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:01</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>70</v>
+        <v>25</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8073,21 +8073,21 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8098,21 +8098,21 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>93</v>
+        <v>32</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,21 +8123,21 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>81</v>
+        <v>36</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,21 +8148,21 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>82</v>
+        <v>40</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8178,16 +8178,16 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8198,21 +8198,21 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8223,21 +8223,21 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>105</v>
+        <v>47</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -8248,21 +8248,21 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>111</v>
+        <v>48</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -8273,21 +8273,21 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>19:36</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>113</v>
+        <v>60</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -8298,23 +8298,248 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
+          <t>18:36:36</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D319" t="n">
+        <v>64</v>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>18:36:36</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>19:41</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D320" t="n">
+        <v>65</v>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>18:36:36</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>19:47</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D321" t="n">
+        <v>71</v>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>18:36:36</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>19:53</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D322" t="n">
+        <v>77</v>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>18:36:36</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>19:54</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D323" t="n">
+        <v>78</v>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
           <t>18:02:23</t>
         </is>
       </c>
-      <c r="B319" t="inlineStr">
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>19:55</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D324" t="n">
+        <v>113</v>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>18:36:36</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
         <is>
           <t>20:00</t>
         </is>
       </c>
-      <c r="C319" t="inlineStr">
+      <c r="C325" t="inlineStr">
         <is>
           <t>81_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D319" t="n">
-        <v>118</v>
-      </c>
-      <c r="E319" t="inlineStr">
+      <c r="D325" t="n">
+        <v>84</v>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>18:36:36</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D326" t="n">
+        <v>99</v>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>18:36:36</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D327" t="n">
+        <v>110</v>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>18:36:36</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D328" t="n">
+        <v>119</v>
+      </c>
+      <c r="E328" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8331,7 +8556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8344,14 +8569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:02:24</t>
+          <t>Última actualización: 18:36:36</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 45</t>
+          <t>Total filas: 46</t>
         </is>
       </c>
     </row>
@@ -9410,7 +9635,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -9420,11 +9645,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -9435,7 +9660,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -9445,11 +9670,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -9460,7 +9685,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -9474,7 +9699,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>82</v>
+        <v>48</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -9485,7 +9710,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -9499,9 +9724,34 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>94</v>
+        <v>60</v>
       </c>
       <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>18:36:36</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>99</v>
+      </c>
+      <c r="E51" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9531,7 +9781,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:02:24</t>
+          <t>Última actualización: 18:36:36</t>
         </is>
       </c>
     </row>
@@ -10722,7 +10972,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -10736,7 +10986,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>76</v>
+        <v>42</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1603
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E328"/>
+  <dimension ref="A1:E336"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:36:36</t>
+          <t>Última actualización: 18:53:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 323</t>
+          <t>Total filas: 331</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2233,11 +2233,11 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>51</v>
+        <v>85</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>85</v>
+        <v>51</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4058,11 +4058,11 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4083,11 +4083,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>2</v>
+        <v>114</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4108,11 +4108,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>114</v>
+        <v>2</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>116</v>
+        <v>28</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>28</v>
+        <v>116</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4733,7 +4733,7 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D176" t="n">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5383,7 +5383,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5408,11 +5408,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -6833,7 +6833,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -6858,7 +6858,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D261" t="n">
@@ -6973,7 +6973,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -6983,11 +6983,11 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>19</v>
+        <v>71</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,7 +6998,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -7008,11 +7008,11 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>71</v>
+        <v>19</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7323,7 +7323,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -7333,11 +7333,11 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>1</v>
+        <v>107</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,7 +7348,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>107</v>
+        <v>1</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,7 +7373,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -7383,11 +7383,11 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,7 +7398,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -7408,11 +7408,11 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7448,7 +7448,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -7458,11 +7458,11 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>13</v>
+        <v>119</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,7 +7473,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -7483,11 +7483,11 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>119</v>
+        <v>13</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7623,7 +7623,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -7633,11 +7633,11 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7798,7 +7798,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
@@ -7808,11 +7808,11 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,7 +7823,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
@@ -7833,11 +7833,11 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7998,7 +7998,7 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
@@ -8012,7 +8012,7 @@
         </is>
       </c>
       <c r="D307" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,7 +8023,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -8037,7 +8037,7 @@
         </is>
       </c>
       <c r="D308" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,7 +8048,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
@@ -8062,7 +8062,7 @@
         </is>
       </c>
       <c r="D309" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8073,12 +8073,12 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>19:04</t>
+          <t>19:03</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
@@ -8087,7 +8087,7 @@
         </is>
       </c>
       <c r="D310" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8103,16 +8103,16 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:04</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,21 +8123,21 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>19:12</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,21 +8148,21 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:12</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8173,12 +8173,12 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -8187,7 +8187,7 @@
         </is>
       </c>
       <c r="D314" t="n">
-        <v>75</v>
+        <v>23</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8198,12 +8198,12 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>19:19</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -8212,7 +8212,7 @@
         </is>
       </c>
       <c r="D315" t="n">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8223,21 +8223,21 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:19</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>47</v>
+        <v>93</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -8248,21 +8248,21 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>48</v>
+        <v>28</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -8273,21 +8273,21 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -8298,21 +8298,21 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>64</v>
+        <v>30</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -8328,16 +8328,16 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,21 +8348,21 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>71</v>
+        <v>42</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8378,16 +8378,16 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:36</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>77</v>
+        <v>60</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -8398,21 +8398,21 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>19:54</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>78</v>
+        <v>47</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -8423,21 +8423,21 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>113</v>
+        <v>65</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -8448,21 +8448,21 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:44</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>84</v>
+        <v>51</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -8473,21 +8473,21 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:47</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>99</v>
+        <v>54</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -8498,21 +8498,21 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>20:26</t>
+          <t>19:53</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>110</v>
+        <v>60</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -8523,23 +8523,223 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
+          <t>18:53:40</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>19:54</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D328" t="n">
+        <v>61</v>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>18:02:23</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>19:55</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D329" t="n">
+        <v>113</v>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>18:53:40</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D330" t="n">
+        <v>67</v>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>18:53:40</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>20:12</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D331" t="n">
+        <v>79</v>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>18:53:40</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D332" t="n">
+        <v>81</v>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
           <t>18:36:36</t>
         </is>
       </c>
-      <c r="B328" t="inlineStr">
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D333" t="n">
+        <v>99</v>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>18:53:40</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D334" t="n">
+        <v>93</v>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>18:53:40</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
         <is>
           <t>20:35</t>
         </is>
       </c>
-      <c r="C328" t="inlineStr">
+      <c r="C335" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D328" t="n">
-        <v>119</v>
-      </c>
-      <c r="E328" t="inlineStr">
+      <c r="D335" t="n">
+        <v>102</v>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>18:53:40</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D336" t="n">
+        <v>111</v>
+      </c>
+      <c r="E336" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8556,7 +8756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8569,14 +8769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:36:36</t>
+          <t>Última actualización: 18:53:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 46</t>
+          <t>Total filas: 50</t>
         </is>
       </c>
     </row>
@@ -9635,7 +9835,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -9645,11 +9845,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -9660,7 +9860,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -9670,11 +9870,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -9685,12 +9885,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>19:24</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -9699,7 +9899,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -9715,16 +9915,16 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:24</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -9735,23 +9935,123 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
+          <t>18:53:40</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>19:35</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>42</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>18:36:36</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>19:36</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>60</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>18:53:40</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>20:14</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>81</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>18:36:36</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
         <is>
           <t>20:15</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C54" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D51" t="n">
+      <c r="D54" t="n">
         <v>99</v>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>18:53:40</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>111</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9768,7 +10068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9781,14 +10081,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:36:36</t>
+          <t>Última actualización: 18:53:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 47</t>
+          <t>Total filas: 49</t>
         </is>
       </c>
     </row>
@@ -10972,25 +11272,75 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
+          <t>18:53:40</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>19:17</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>24</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
           <t>18:36:36</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>19:18</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D52" t="n">
+      <c r="D53" t="n">
         <v>42</v>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>18:53:40</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>111</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1604
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E336"/>
+  <dimension ref="A1:E342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:53:40</t>
+          <t>Última actualización: 19:14:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 331</t>
+          <t>Total filas: 337</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,7 +2973,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -2983,11 +2983,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>97</v>
+        <v>3</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>3</v>
+        <v>97</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -4333,11 +4333,11 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>40</v>
+        <v>16</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -5383,7 +5383,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -5408,7 +5408,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7323,7 +7323,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -7333,11 +7333,11 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>107</v>
+        <v>1</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,7 +7348,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>1</v>
+        <v>107</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,7 +7373,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -7383,11 +7383,11 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,7 +7398,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -7408,11 +7408,11 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7623,7 +7623,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -7633,11 +7633,11 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>80</v>
+        <v>26</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7798,7 +7798,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
@@ -7808,11 +7808,11 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,7 +7823,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
@@ -7833,11 +7833,11 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -8173,7 +8173,7 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
@@ -8187,7 +8187,7 @@
         </is>
       </c>
       <c r="D314" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8248,7 +8248,7 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
@@ -8262,7 +8262,7 @@
         </is>
       </c>
       <c r="D317" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -8298,7 +8298,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
@@ -8312,7 +8312,7 @@
         </is>
       </c>
       <c r="D319" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -8323,7 +8323,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -8337,7 +8337,7 @@
         </is>
       </c>
       <c r="D320" t="n">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,21 +8348,21 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>19:35</t>
+          <t>19:33</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8373,12 +8373,12 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>19:36</t>
+          <t>19:35</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -8387,7 +8387,7 @@
         </is>
       </c>
       <c r="D322" t="n">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -8398,21 +8398,21 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:36</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>47</v>
+        <v>22</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -8423,21 +8423,21 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>65</v>
+        <v>26</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -8448,12 +8448,12 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>19:44</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -8462,7 +8462,7 @@
         </is>
       </c>
       <c r="D325" t="n">
-        <v>51</v>
+        <v>65</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -8473,21 +8473,21 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>19:47</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -8503,16 +8503,16 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>19:53</t>
+          <t>19:44</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -8523,21 +8523,21 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>19:54</t>
+          <t>19:47</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -8548,21 +8548,21 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>19:55</t>
+          <t>19:53</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>113</v>
+        <v>39</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -8573,21 +8573,21 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>19:54</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>67</v>
+        <v>40</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -8598,21 +8598,21 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>18:02:23</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>20:12</t>
+          <t>19:55</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -8623,21 +8623,21 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:00</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -8648,21 +8648,21 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:11</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>99</v>
+        <v>57</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -8678,16 +8678,16 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>20:26</t>
+          <t>20:12</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8703,16 +8703,16 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>102</v>
+        <v>81</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,23 +8723,173 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D336" t="n">
+        <v>61</v>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>19:14:28</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>20:26</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D337" t="n">
+        <v>72</v>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>19:14:28</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D338" t="n">
+        <v>81</v>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>19:14:28</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
           <t>20:44</t>
         </is>
       </c>
-      <c r="C336" t="inlineStr">
+      <c r="C339" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D336" t="n">
-        <v>111</v>
-      </c>
-      <c r="E336" t="inlineStr">
+      <c r="D339" t="n">
+        <v>90</v>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>19:14:28</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D340" t="n">
+        <v>101</v>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>19:14:28</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D341" t="n">
+        <v>101</v>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>19:14:28</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D342" t="n">
+        <v>102</v>
+      </c>
+      <c r="E342" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8756,7 +8906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8769,14 +8919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:53:40</t>
+          <t>Última actualización: 19:14:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 50</t>
+          <t>Total filas: 51</t>
         </is>
       </c>
     </row>
@@ -9910,7 +10060,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -9924,7 +10074,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>48</v>
+        <v>10</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -9960,7 +10110,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -9974,7 +10124,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -10010,7 +10160,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -10024,7 +10174,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>99</v>
+        <v>61</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -10035,7 +10185,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -10049,9 +10199,34 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>111</v>
+        <v>90</v>
       </c>
       <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>19:14:28</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>101</v>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10068,7 +10243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10081,14 +10256,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:53:40</t>
+          <t>Última actualización: 19:14:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 49</t>
+          <t>Total filas: 51</t>
         </is>
       </c>
     </row>
@@ -11272,12 +11447,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>19:17</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -11286,7 +11461,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -11297,12 +11472,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>19:18</t>
+          <t>19:17</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -11311,7 +11486,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -11322,23 +11497,73 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>18:36:36</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>42</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
           <t>18:53:40</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>20:44</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D54" t="n">
+      <c r="D55" t="n">
         <v>111</v>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>19:14:28</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>91</v>
+      </c>
+      <c r="E56" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1605
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E342"/>
+  <dimension ref="A1:E351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:14:28</t>
+          <t>Última actualización: 19:46:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 337</t>
+          <t>Total filas: 346</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>07:16:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07:16:54</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2233,11 +2233,11 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>85</v>
+        <v>51</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>51</v>
+        <v>85</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4058,11 +4058,11 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>28</v>
+        <v>116</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>116</v>
+        <v>28</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>95</v>
+        <v>17</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>17</v>
+        <v>95</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4683,11 +4683,11 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -6883,7 +6883,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D262" t="n">
@@ -6908,7 +6908,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D263" t="n">
@@ -7623,7 +7623,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -7633,11 +7633,11 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>80</v>
+        <v>26</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7798,7 +7798,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
@@ -7808,11 +7808,11 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,7 +7823,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
@@ -7833,11 +7833,11 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -8448,7 +8448,7 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
@@ -8458,11 +8458,11 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>65</v>
+        <v>27</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -8473,7 +8473,7 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
@@ -8483,11 +8483,11 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>27</v>
+        <v>65</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -8523,7 +8523,7 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>19:46:17</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
@@ -8537,7 +8537,7 @@
         </is>
       </c>
       <c r="D328" t="n">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -8548,7 +8548,7 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>19:46:17</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
@@ -8562,7 +8562,7 @@
         </is>
       </c>
       <c r="D329" t="n">
-        <v>39</v>
+        <v>7</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -8598,7 +8598,7 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>18:02:23</t>
+          <t>19:46:17</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
@@ -8612,7 +8612,7 @@
         </is>
       </c>
       <c r="D331" t="n">
-        <v>113</v>
+        <v>9</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -8623,7 +8623,7 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>19:46:17</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
@@ -8637,7 +8637,7 @@
         </is>
       </c>
       <c r="D332" t="n">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -8648,21 +8648,21 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>19:46:17</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>20:11</t>
+          <t>20:07</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -8673,12 +8673,12 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:46:17</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>20:12</t>
+          <t>20:11</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -8687,7 +8687,7 @@
         </is>
       </c>
       <c r="D334" t="n">
-        <v>79</v>
+        <v>25</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8698,21 +8698,21 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:46:17</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:11</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>81</v>
+        <v>25</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,21 +8723,21 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:12</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,21 +8748,21 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>20:26</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -8773,21 +8773,21 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>19:46:17</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>81</v>
+        <v>29</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8803,16 +8803,16 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:26</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8823,21 +8823,21 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>19:46:17</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:27</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>101</v>
+        <v>41</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -8848,21 +8848,21 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>19:46:17</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:32</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>101</v>
+        <v>46</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,23 +8873,248 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
+          <t>19:46:17</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>20:35</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D342" t="n">
+        <v>49</v>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>19:46:17</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>20:44</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D343" t="n">
+        <v>58</v>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
           <t>19:14:28</t>
         </is>
       </c>
-      <c r="B342" t="inlineStr">
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D344" t="n">
+        <v>101</v>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>19:14:28</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>20:55</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D345" t="n">
+        <v>101</v>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>19:46:17</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
         <is>
           <t>20:56</t>
         </is>
       </c>
-      <c r="C342" t="inlineStr">
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D346" t="n">
+        <v>70</v>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>19:14:28</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D342" t="n">
+      <c r="D347" t="n">
         <v>102</v>
       </c>
-      <c r="E342" t="inlineStr">
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>19:46:17</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>20:58</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D348" t="n">
+        <v>72</v>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>19:46:17</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>21:01</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D349" t="n">
+        <v>75</v>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>19:46:17</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>21:24</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D350" t="n">
+        <v>98</v>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>19:46:17</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D351" t="n">
+        <v>99</v>
+      </c>
+      <c r="E351" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8906,7 +9131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8919,14 +9144,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:14:28</t>
+          <t>Última actualización: 19:46:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 51</t>
+          <t>Total filas: 52</t>
         </is>
       </c>
     </row>
@@ -10160,7 +10385,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>19:46:17</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -10174,7 +10399,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -10185,7 +10410,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>19:46:17</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -10199,7 +10424,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>90</v>
+        <v>58</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -10227,6 +10452,31 @@
         <v>101</v>
       </c>
       <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>19:46:17</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>20:56</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>70</v>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10243,7 +10493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E56"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10256,14 +10506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:14:28</t>
+          <t>Última actualización: 19:46:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 51</t>
+          <t>Total filas: 52</t>
         </is>
       </c>
     </row>
@@ -11547,7 +11797,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>19:46:17</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -11561,9 +11811,34 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>91</v>
+        <v>59</v>
       </c>
       <c r="E56" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>19:46:17</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>21:37</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>111</v>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1606
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E351"/>
+  <dimension ref="A1:E356"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:46:17</t>
+          <t>Última actualización: 20:02:17</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 346</t>
+          <t>Total filas: 351</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,7 +2498,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2508,11 +2508,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>16</v>
+        <v>50</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4058,11 +4058,11 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4083,11 +4083,11 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>114</v>
+        <v>2</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4108,11 +4108,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>2</v>
+        <v>114</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>17</v>
+        <v>95</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>95</v>
+        <v>17</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5408,11 +5408,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -6833,7 +6833,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -6858,7 +6858,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D261" t="n">
@@ -6973,7 +6973,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -6983,11 +6983,11 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>71</v>
+        <v>19</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,7 +6998,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -7008,11 +7008,11 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>19</v>
+        <v>71</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7323,7 +7323,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -7333,11 +7333,11 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>1</v>
+        <v>107</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,7 +7348,7 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
@@ -7358,11 +7358,11 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>107</v>
+        <v>1</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,7 +7373,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -7383,11 +7383,11 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,7 +7398,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -7408,11 +7408,11 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7623,7 +7623,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -7633,11 +7633,11 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>26</v>
+        <v>80</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7798,7 +7798,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
@@ -7808,11 +7808,11 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7848,7 +7848,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
@@ -7858,11 +7858,11 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -8273,7 +8273,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
@@ -8283,11 +8283,11 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -8298,7 +8298,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
@@ -8308,11 +8308,11 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -8448,7 +8448,7 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
@@ -8458,11 +8458,11 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>27</v>
+        <v>65</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -8473,7 +8473,7 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
@@ -8483,11 +8483,11 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>65</v>
+        <v>27</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -8648,7 +8648,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
@@ -8662,7 +8662,7 @@
         </is>
       </c>
       <c r="D333" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -8673,7 +8673,7 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
@@ -8687,7 +8687,7 @@
         </is>
       </c>
       <c r="D334" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8723,7 +8723,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
@@ -8733,11 +8733,11 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8753,16 +8753,16 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>20:14</t>
+          <t>20:12</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -8773,12 +8773,12 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:14</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -8787,7 +8787,7 @@
         </is>
       </c>
       <c r="D338" t="n">
-        <v>29</v>
+        <v>81</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,21 +8798,21 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>20:26</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>72</v>
+        <v>13</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8823,12 +8823,12 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>20:27</t>
+          <t>20:26</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -8837,7 +8837,7 @@
         </is>
       </c>
       <c r="D340" t="n">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -8848,21 +8848,21 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>20:32</t>
+          <t>20:27</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,21 +8873,21 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>20:35</t>
+          <t>20:32</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>49</v>
+        <v>30</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -8898,21 +8898,21 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>20:44</t>
+          <t>20:35</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -8923,21 +8923,21 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:44</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>101</v>
+        <v>42</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8973,21 +8973,21 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>70</v>
+        <v>101</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,7 +8998,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
@@ -9008,11 +9008,11 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>102</v>
+        <v>54</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9023,12 +9023,12 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>20:58</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -9037,7 +9037,7 @@
         </is>
       </c>
       <c r="D348" t="n">
-        <v>72</v>
+        <v>102</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -9048,21 +9048,21 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>21:01</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9078,16 +9078,16 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>21:24</t>
+          <t>20:58</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>98</v>
+        <v>72</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9098,23 +9098,148 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
+          <t>20:02:17</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>20:59</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D351" t="n">
+        <v>57</v>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
           <t>19:46:17</t>
         </is>
       </c>
-      <c r="B351" t="inlineStr">
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>21:01</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D352" t="n">
+        <v>75</v>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>20:02:17</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>21:24</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D353" t="n">
+        <v>82</v>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>20:02:17</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
         <is>
           <t>21:25</t>
         </is>
       </c>
-      <c r="C351" t="inlineStr">
+      <c r="C354" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D351" t="n">
-        <v>99</v>
-      </c>
-      <c r="E351" t="inlineStr">
+      <c r="D354" t="n">
+        <v>83</v>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>20:02:17</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D355" t="n">
+        <v>107</v>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>20:02:17</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>21:50</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>108</v>
+      </c>
+      <c r="E356" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9144,7 +9269,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:46:17</t>
+          <t>Última actualización: 20:02:17</t>
         </is>
       </c>
     </row>
@@ -10385,7 +10510,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -10399,7 +10524,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -10410,7 +10535,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -10424,7 +10549,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -10460,7 +10585,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -10474,7 +10599,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -10506,7 +10631,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:46:17</t>
+          <t>Última actualización: 20:02:17</t>
         </is>
       </c>
     </row>
@@ -11797,7 +11922,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -11811,7 +11936,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -11822,7 +11947,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -11836,7 +11961,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>111</v>
+        <v>95</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1607
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E356"/>
+  <dimension ref="A1:E362"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:02:17</t>
+          <t>Última actualización: 20:38:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 351</t>
+          <t>Total filas: 357</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -2948,7 +2948,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -2958,11 +2958,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>8</v>
+        <v>68</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3248,7 +3248,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -3258,11 +3258,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>3</v>
+        <v>97</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,7 +3273,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -3283,11 +3283,11 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>97</v>
+        <v>3</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4058,11 +4058,11 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>116</v>
+        <v>28</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>28</v>
+        <v>116</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>95</v>
+        <v>17</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>17</v>
+        <v>95</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5383,7 +5383,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5408,11 +5408,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:50:32</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:50:32</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5758,11 +5758,11 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -6833,7 +6833,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -6858,7 +6858,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D261" t="n">
@@ -6883,7 +6883,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D262" t="n">
@@ -6908,7 +6908,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D263" t="n">
@@ -6973,7 +6973,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -6983,11 +6983,11 @@
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>19</v>
+        <v>71</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,7 +6998,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -7008,11 +7008,11 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>71</v>
+        <v>19</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7373,7 +7373,7 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
@@ -7383,11 +7383,11 @@
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,7 +7398,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
@@ -7408,11 +7408,11 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7448,7 +7448,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -7458,11 +7458,11 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>119</v>
+        <v>13</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,7 +7473,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -7483,11 +7483,11 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>13</v>
+        <v>119</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7808,7 +7808,7 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D299" t="n">
@@ -7833,7 +7833,7 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D300" t="n">
@@ -8923,7 +8923,7 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>20:02:17</t>
+          <t>20:38:03</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
@@ -8937,7 +8937,7 @@
         </is>
       </c>
       <c r="D344" t="n">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8948,21 +8948,21 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>20:38:03</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>20:55</t>
+          <t>20:50</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>101</v>
+        <v>12</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8998,12 +8998,12 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>20:02:17</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>20:56</t>
+          <t>20:55</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -9012,7 +9012,7 @@
         </is>
       </c>
       <c r="D347" t="n">
-        <v>54</v>
+        <v>101</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9048,21 +9048,21 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>20:02:17</t>
+          <t>20:38:03</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>20:57</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>55</v>
+        <v>18</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9073,21 +9073,21 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>20:38:03</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>20:58</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>72</v>
+        <v>18</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9098,21 +9098,21 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>20:02:17</t>
+          <t>20:38:03</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>20:59</t>
+          <t>20:57</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>57</v>
+        <v>19</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9128,16 +9128,16 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>21:01</t>
+          <t>20:58</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -9153,16 +9153,16 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>21:24</t>
+          <t>20:59</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>82</v>
+        <v>57</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -9173,21 +9173,21 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>20:02:17</t>
+          <t>19:46:17</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>21:25</t>
+          <t>21:01</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -9198,21 +9198,21 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>20:02:17</t>
+          <t>20:38:03</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>21:22</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>107</v>
+        <v>44</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -9223,23 +9223,173 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>20:02:17</t>
+          <t>20:38:03</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
+          <t>21:24</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>46</v>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>20:38:03</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D357" t="n">
+        <v>47</v>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>20:38:03</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>21:43</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D358" t="n">
+        <v>65</v>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>20:38:03</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D359" t="n">
+        <v>71</v>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>20:38:03</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
           <t>21:50</t>
         </is>
       </c>
-      <c r="C356" t="inlineStr">
+      <c r="C360" t="inlineStr">
         <is>
           <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
-      <c r="D356" t="n">
-        <v>108</v>
-      </c>
-      <c r="E356" t="inlineStr">
+      <c r="D360" t="n">
+        <v>72</v>
+      </c>
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>20:38:03</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>22:19</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D361" t="n">
+        <v>101</v>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>20:38:03</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>22:27</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D362" t="n">
+        <v>109</v>
+      </c>
+      <c r="E362" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9256,7 +9406,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9269,14 +9419,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:02:17</t>
+          <t>Última actualización: 20:38:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 52</t>
+          <t>Total filas: 53</t>
         </is>
       </c>
     </row>
@@ -10535,7 +10685,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>20:02:17</t>
+          <t>20:38:03</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -10549,7 +10699,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -10585,7 +10735,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>20:02:17</t>
+          <t>20:38:03</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -10599,9 +10749,34 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>54</v>
+        <v>18</v>
       </c>
       <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>20:38:03</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>22:27</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>109</v>
+      </c>
+      <c r="E58" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10618,7 +10793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10631,14 +10806,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:02:17</t>
+          <t>Última actualización: 20:38:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 52</t>
+          <t>Total filas: 55</t>
         </is>
       </c>
     </row>
@@ -11947,25 +12122,100 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>20:02:17</t>
+          <t>20:38:03</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
+          <t>20:46</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>8</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>20:38:03</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
           <t>21:37</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D57" t="n">
-        <v>95</v>
-      </c>
-      <c r="E57" t="inlineStr">
+      <c r="D58" t="n">
+        <v>59</v>
+      </c>
+      <c r="E58" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>20:38:03</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>94</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>20:38:03</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>22:32</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>114</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1608
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E362"/>
+  <dimension ref="A1:E368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:38:03</t>
+          <t>Última actualización: 20:55:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 357</t>
+          <t>Total filas: 363</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1708,7 +1708,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -1733,7 +1733,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2233,11 +2233,11 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2983,7 +2983,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D106" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D107" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3533,7 +3533,7 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D128" t="n">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D129" t="n">
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>17</v>
+        <v>95</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>95</v>
+        <v>17</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4708,7 +4708,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
@@ -4983,7 +4983,7 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D186" t="n">
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D200" t="n">
@@ -5383,7 +5383,7 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D202" t="n">
@@ -5408,7 +5408,7 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D203" t="n">
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7448,7 +7448,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -7458,11 +7458,11 @@
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>13</v>
+        <v>119</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,7 +7473,7 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
@@ -7483,11 +7483,11 @@
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>119</v>
+        <v>13</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7823,7 +7823,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
@@ -7833,11 +7833,11 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,7 +7848,7 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
@@ -7858,11 +7858,11 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -8273,7 +8273,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
@@ -8283,11 +8283,11 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -8298,7 +8298,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
@@ -8308,11 +8308,11 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -8673,7 +8673,7 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>20:02:17</t>
+          <t>19:46:17</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
@@ -8683,11 +8683,11 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8698,7 +8698,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
@@ -8708,11 +8708,11 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,7 +8723,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>20:02:17</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
@@ -8733,11 +8733,11 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,7 +8748,7 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
@@ -8758,11 +8758,11 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -8973,7 +8973,7 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>20:55:37</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
@@ -8983,11 +8983,11 @@
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>101</v>
+        <v>0</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -9008,7 +9008,7 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D347" t="n">
@@ -9023,7 +9023,7 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>20:38:03</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
@@ -9033,11 +9033,11 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>102</v>
+        <v>18</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -9073,7 +9073,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>20:38:03</t>
+          <t>20:55:37</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -9083,11 +9083,11 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9198,7 +9198,7 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>20:38:03</t>
+          <t>20:55:37</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
@@ -9212,7 +9212,7 @@
         </is>
       </c>
       <c r="D355" t="n">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -9223,12 +9223,12 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>20:38:03</t>
+          <t>20:55:37</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>21:24</t>
+          <t>21:23</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -9237,7 +9237,7 @@
         </is>
       </c>
       <c r="D356" t="n">
-        <v>46</v>
+        <v>28</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -9253,16 +9253,16 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>21:25</t>
+          <t>21:24</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -9273,21 +9273,21 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>20:38:03</t>
+          <t>20:55:37</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>21:43</t>
+          <t>21:25</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>65</v>
+        <v>30</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -9303,16 +9303,16 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>21:49</t>
+          <t>21:43</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -9323,21 +9323,21 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>20:38:03</t>
+          <t>20:55:37</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>21:50</t>
+          <t>21:47</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>72</v>
+        <v>52</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -9348,21 +9348,21 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>20:38:03</t>
+          <t>20:55:37</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>22:19</t>
+          <t>21:47</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D361" t="n">
-        <v>101</v>
+        <v>52</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -9373,23 +9373,173 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
+          <t>20:55:37</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>21:49</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D362" t="n">
+        <v>54</v>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>20:55:37</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>21:50</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D363" t="n">
+        <v>55</v>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>20:55:37</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>22:19</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D364" t="n">
+        <v>84</v>
+      </c>
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>20:55:37</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>22:22</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D365" t="n">
+        <v>87</v>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>20:55:37</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D366" t="n">
+        <v>91</v>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
           <t>20:38:03</t>
         </is>
       </c>
-      <c r="B362" t="inlineStr">
+      <c r="B367" t="inlineStr">
         <is>
           <t>22:27</t>
         </is>
       </c>
-      <c r="C362" t="inlineStr">
+      <c r="C367" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D362" t="n">
+      <c r="D367" t="n">
         <v>109</v>
       </c>
-      <c r="E362" t="inlineStr">
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>20:55:37</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>22:49</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D368" t="n">
+        <v>114</v>
+      </c>
+      <c r="E368" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9406,7 +9556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9419,14 +9569,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:38:03</t>
+          <t>Última actualización: 20:55:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 53</t>
+          <t>Total filas: 54</t>
         </is>
       </c>
     </row>
@@ -10435,7 +10585,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -10445,11 +10595,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1</v>
+        <v>107</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -10460,7 +10610,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -10470,11 +10620,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>107</v>
+        <v>1</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -10485,7 +10635,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -10495,11 +10645,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -10510,7 +10660,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -10520,11 +10670,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -10710,7 +10860,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>20:55:37</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -10724,7 +10874,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>101</v>
+        <v>0</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -10760,23 +10910,48 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>20:55:37</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>91</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>20:38:03</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>22:27</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D58" t="n">
+      <c r="D59" t="n">
         <v>109</v>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10793,7 +10968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10806,14 +10981,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:38:03</t>
+          <t>Última actualización: 20:55:37</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 55</t>
+          <t>Total filas: 56</t>
         </is>
       </c>
     </row>
@@ -12172,48 +12347,73 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>20:38:03</t>
+          <t>20:55:37</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>22:12</t>
+          <t>21:38</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>94</v>
+        <v>43</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>20:38:03</t>
+          <t>20:55:37</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
+          <t>22:12</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>77</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>20:55:37</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
           <t>22:32</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D60" t="n">
-        <v>114</v>
-      </c>
-      <c r="E60" t="inlineStr">
+      <c r="D61" t="n">
+        <v>97</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 1609
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-03-14.xlsx
+++ b/data/horarios-141-2026-03-14.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E368"/>
+  <dimension ref="A1:E378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:55:37</t>
+          <t>Última actualización: 22:17:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 363</t>
+          <t>Total filas: 373</t>
         </is>
       </c>
     </row>
@@ -633,7 +633,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -658,7 +658,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -683,7 +683,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1858,7 +1858,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>08:02:29</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1933,11 +1933,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>9</v>
+        <v>58</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>08:02:29</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>58</v>
+        <v>9</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>07:48:06</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2233,11 +2233,11 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>07:48:06</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:51:02</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>9</v>
+        <v>43</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:51:02</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>43</v>
+        <v>9</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2698,7 +2698,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>09:25:12</t>
+          <t>08:33:50</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>38</v>
+        <v>90</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,7 +2723,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:33:50</t>
+          <t>09:25:12</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2733,11 +2733,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>90</v>
+        <v>38</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -2908,7 +2908,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3623,7 +3623,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -3633,11 +3633,11 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>34</v>
+        <v>5</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3658,11 +3658,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>5</v>
+        <v>34</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>51</v>
+        <v>85</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,7 +3773,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -3783,11 +3783,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>85</v>
+        <v>51</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3898,7 +3898,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>10</v>
+        <v>98</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,7 +3923,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -3933,11 +3933,11 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>98</v>
+        <v>10</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,7 +3948,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -3958,11 +3958,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>11</v>
+        <v>65</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,7 +3973,7 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>65</v>
+        <v>11</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>11:28:56</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -4033,11 +4033,11 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,7 +4048,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>11:28:56</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -4058,11 +4058,11 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4123,7 +4123,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>11:53:49</t>
+          <t>10:25:57</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>28</v>
+        <v>116</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:25:57</t>
+          <t>11:53:49</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4158,11 +4158,11 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>116</v>
+        <v>28</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4348,7 +4348,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>10:59:29</t>
+          <t>12:17:07</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>95</v>
+        <v>17</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>12:17:07</t>
+          <t>10:59:29</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4383,11 +4383,11 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>17</v>
+        <v>95</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:59:51</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4708,11 +4708,11 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,7 +4723,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>12:59:51</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -4733,11 +4733,11 @@
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>12:45:09</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5008,11 +5008,11 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>52</v>
+        <v>4</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>12:45:09</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5033,11 +5033,11 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>4</v>
+        <v>52</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>13:33:52</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5358,11 +5358,11 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>13:33:52</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5408,11 +5408,11 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>17</v>
+        <v>44</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>14:27:41</t>
+          <t>14:00:00</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5533,11 +5533,11 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>6</v>
+        <v>33</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>14:00:00</t>
+          <t>14:27:41</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5558,11 +5558,11 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>33</v>
+        <v>6</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -6508,7 +6508,7 @@
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215_ALUAR</t>
         </is>
       </c>
       <c r="D247" t="n">
@@ -6533,7 +6533,7 @@
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>215_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -6583,7 +6583,7 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -6608,7 +6608,7 @@
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -6833,7 +6833,7 @@
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D260" t="n">
@@ -6858,7 +6858,7 @@
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D261" t="n">
@@ -6883,7 +6883,7 @@
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D262" t="n">
@@ -6908,7 +6908,7 @@
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D263" t="n">
@@ -7158,7 +7158,7 @@
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D273" t="n">
@@ -7183,7 +7183,7 @@
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D274" t="n">
@@ -7623,7 +7623,7 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>17:15:35</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
@@ -7633,11 +7633,11 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>57</v>
+        <v>26</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>16:52:15</t>
+          <t>17:15:35</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>80</v>
+        <v>57</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:52:15</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>26</v>
+        <v>80</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7798,7 +7798,7 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
@@ -7808,11 +7808,11 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,7 +7823,7 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
@@ -7833,11 +7833,11 @@
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7858,7 +7858,7 @@
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D301" t="n">
@@ -8273,7 +8273,7 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
@@ -8283,11 +8283,11 @@
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -8298,7 +8298,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
@@ -8308,11 +8308,11 @@
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -8448,7 +8448,7 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>18:36:36</t>
+          <t>19:14:28</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
@@ -8458,11 +8458,11 @@
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>65</v>
+        <v>27</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -8473,7 +8473,7 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>19:14:28</t>
+          <t>18:36:36</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
@@ -8483,11 +8483,11 @@
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>27</v>
+        <v>65</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -8673,7 +8673,7 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>19:46:17</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
@@ -8683,11 +8683,11 @@
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>25</v>
+        <v>9</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8698,7 +8698,7 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>20:02:17</t>
+          <t>19:46:17</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
@@ -8708,11 +8708,11 @@
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,7 +8723,7 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>18:53:40</t>
+          <t>20:02:17</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
@@ -8733,11 +8733,11 @@
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>79</v>
+        <v>10</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,7 +8748,7 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>20:02:17</t>
+          <t>18:53:40</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
@@ -8758,11 +8758,11 @@
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>10</v>
+        <v>79</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -9033,7 +9033,7 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D348" t="n">
@@ -9048,7 +9048,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>20:38:03</t>
+          <t>20:55:37</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
@@ -9058,11 +9058,11 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9073,7 +9073,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>20:55:37</t>
+          <t>20:38:03</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -9083,11 +9083,11 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9333,7 +9333,7 @@
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D360" t="n">
@@ -9358,7 +9358,7 @@
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D361" t="n">
@@ -9423,12 +9423,12 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>20:55:37</t>
+          <t>22:17:53</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>22:19</t>
+          <t>22:17</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -9437,7 +9437,7 @@
         </is>
       </c>
       <c r="D364" t="n">
-        <v>84</v>
+        <v>0</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -9448,21 +9448,21 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>20:55:37</t>
+          <t>22:17:53</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>22:22</t>
+          <t>22:17</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D365" t="n">
-        <v>87</v>
+        <v>0</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -9473,21 +9473,21 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>20:55:37</t>
+          <t>22:17:53</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>22:26</t>
+          <t>22:17</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>91</v>
+        <v>0</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -9498,21 +9498,21 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>20:38:03</t>
+          <t>20:55:37</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>22:27</t>
+          <t>22:19</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D367" t="n">
-        <v>109</v>
+        <v>84</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -9528,18 +9528,268 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
+          <t>22:22</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D368" t="n">
+        <v>87</v>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>22:17:53</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>22:26</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D369" t="n">
+        <v>9</v>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>20:38:03</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>22:27</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D370" t="n">
+        <v>109</v>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>22:17:53</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>22:48</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D371" t="n">
+        <v>31</v>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>20:55:37</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
           <t>22:49</t>
         </is>
       </c>
-      <c r="C368" t="inlineStr">
+      <c r="C372" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D368" t="n">
+      <c r="D372" t="n">
         <v>114</v>
       </c>
-      <c r="E368" t="inlineStr">
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>22:17:53</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>22:58</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D373" t="n">
+        <v>41</v>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>22:17:53</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>23:12</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D374" t="n">
+        <v>55</v>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>22:17:53</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>23:18</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D375" t="n">
+        <v>61</v>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>22:17:53</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>23:28</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D376" t="n">
+        <v>71</v>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>22:17:53</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>23:48</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D377" t="n">
+        <v>91</v>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>22:17:53</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>23:54</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D378" t="n">
+        <v>97</v>
+      </c>
+      <c r="E378" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9556,7 +9806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9569,14 +9819,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:55:37</t>
+          <t>Última actualización: 22:17:53</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 54</t>
+          <t>Total filas: 55</t>
         </is>
       </c>
     </row>
@@ -10585,7 +10835,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>16:00:50</t>
+          <t>17:46:20</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -10595,11 +10845,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>107</v>
+        <v>1</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -10610,7 +10860,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>17:46:20</t>
+          <t>16:00:50</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -10620,11 +10870,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>1</v>
+        <v>107</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -10910,7 +11160,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>20:55:37</t>
+          <t>22:17:53</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -10924,7 +11174,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>91</v>
+        <v>9</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -10952,6 +11202,31 @@
         <v>109</v>
       </c>
       <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>22:17:53</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>23:54</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>97</v>
+      </c>
+      <c r="E60" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10981,7 +11256,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:55:37</t>
+          <t>Última actualización: 22:17:53</t>
         </is>
       </c>
     </row>
@@ -12397,7 +12672,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>20:55:37</t>
+          <t>22:17:53</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -12411,7 +12686,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>97</v>
+        <v>15</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>

</xml_diff>